<commit_message>
- add animation on every move - remove room.red_first field which comes from xiangqi - enhace responisive experience - config backend port for deployment
</commit_message>
<xml_diff>
--- a/tools/languages.xlsx
+++ b/tools/languages.xlsx
@@ -325,7 +325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C472"/>
+  <dimension ref="A1:C471"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3855,4184 +3855,4172 @@
     <row r="208" ht="18" customHeight="1">
       <c r="A208" s="1" t="inlineStr">
         <is>
-          <t>create-room.messages.invalid-redFirst</t>
+          <t>create-room.messages.invalid-team-name</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>'redFirst' must be a boolean</t>
+          <t>Team name must be either 'red', 'black', or null</t>
         </is>
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>'redFirst' phải là giá trị boolean</t>
+          <t>Tên đội phải là 'red', 'black' hoặc null</t>
         </is>
       </c>
     </row>
     <row r="209" ht="18" customHeight="1">
       <c r="A209" s="1" t="inlineStr">
         <is>
-          <t>create-room.messages.invalid-team-name</t>
+          <t>create-room.messages.name-required</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>Team name must be either 'red', 'black', or null</t>
+          <t>Room name (tableName) is required and must not be empty</t>
         </is>
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>Tên đội phải là 'red', 'black' hoặc null</t>
+          <t>Tên phòng (tableName) là bắt buộc và không được để trống</t>
         </is>
       </c>
     </row>
     <row r="210" ht="18" customHeight="1">
       <c r="A210" s="1" t="inlineStr">
         <is>
-          <t>create-room.messages.name-required</t>
+          <t>create-room.messages.room-created</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>Room name (tableName) is required and must not be empty</t>
+          <t>Room created successfully</t>
         </is>
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>Tên phòng (tableName) là bắt buộc và không được để trống</t>
+          <t>Phòng được tạo thành công</t>
         </is>
       </c>
     </row>
     <row r="211" ht="36" customHeight="1">
       <c r="A211" s="1" t="inlineStr">
         <is>
-          <t>create-room.messages.room-created</t>
+          <t>fetch-rooms.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>Room created successfully</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>Phòng được tạo thành công</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="212" ht="18" customHeight="1">
       <c r="A212" s="1" t="inlineStr">
         <is>
-          <t>fetch-rooms.messages.internal-server-error</t>
+          <t>fetch-rooms.messages.invalid-status</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Query parameter 'status' must be an integer</t>
         </is>
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Tham số truy vấn 'status' phải là số nguyên</t>
         </is>
       </c>
     </row>
     <row r="213" ht="18" customHeight="1">
       <c r="A213" s="1" t="inlineStr">
         <is>
-          <t>fetch-rooms.messages.invalid-status</t>
+          <t>fetch-rooms.messages.success</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>Query parameter 'status' must be an integer</t>
+          <t>Fetch rooms successfully</t>
         </is>
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>Tham số truy vấn 'status' phải là số nguyên</t>
+          <t>Lấy phòng thành công</t>
         </is>
       </c>
     </row>
     <row r="214" ht="18" customHeight="1">
       <c r="A214" s="1" t="inlineStr">
         <is>
-          <t>fetch-rooms.messages.success</t>
+          <t>forgot-password.messages.email-not-found</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>Fetch rooms successfully</t>
+          <t>Email does not exist</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>Lấy phòng thành công</t>
+          <t>Email không tồn tại</t>
         </is>
       </c>
     </row>
     <row r="215" ht="18" customHeight="1">
       <c r="A215" s="1" t="inlineStr">
         <is>
-          <t>forgot-password.messages.email-not-found</t>
+          <t>forgot-password.messages.email-service-not-configured</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>Email does not exist</t>
+          <t>Email service is not configured</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>Email không tồn tại</t>
+          <t>Dịch vụ email chưa được cấu hình</t>
         </is>
       </c>
     </row>
     <row r="216" ht="18" customHeight="1">
       <c r="A216" s="1" t="inlineStr">
         <is>
-          <t>forgot-password.messages.email-service-not-configured</t>
+          <t>forgot-password.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>Email service is not configured</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>Dịch vụ email chưa được cấu hình</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="217" ht="18" customHeight="1">
       <c r="A217" s="1" t="inlineStr">
         <is>
-          <t>forgot-password.messages.internal-server-error</t>
+          <t>forgot-password.messages.invalid-email-format</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Invalid email format</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Định dạng email không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="218" ht="18" customHeight="1">
       <c r="A218" s="1" t="inlineStr">
         <is>
-          <t>forgot-password.messages.invalid-email-format</t>
+          <t>forgot-password.messages.missing-email</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>Invalid email format</t>
+          <t>Email is required</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>Định dạng email không hợp lệ</t>
+          <t>Email là bắt buộc</t>
         </is>
       </c>
     </row>
     <row r="219" ht="18" customHeight="1">
       <c r="A219" s="1" t="inlineStr">
         <is>
-          <t>forgot-password.messages.missing-email</t>
+          <t>forgot-password.messages.success</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
         <is>
-          <t>Email is required</t>
+          <t>Forgot password email sent</t>
         </is>
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>Email là bắt buộc</t>
+          <t>Email đặt lại mật khẩu đã được gửi</t>
         </is>
       </c>
     </row>
     <row r="220" ht="18" customHeight="1">
       <c r="A220" s="1" t="inlineStr">
         <is>
-          <t>forgot-password.messages.success</t>
+          <t>join-room.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t>Forgot password email sent</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Email đặt lại mật khẩu đã được gửi</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="221" ht="18" customHeight="1">
       <c r="A221" s="1" t="inlineStr">
         <is>
-          <t>join-room.messages.internal-server-error</t>
+          <t>join-room.messages.invalid-team</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Field 'team' must be 'red', 'black', null, or undefined</t>
         </is>
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Trường 'team' phải là 'red', 'black', null hoặc không truyền</t>
         </is>
       </c>
     </row>
     <row r="222" ht="18" customHeight="1">
       <c r="A222" s="1" t="inlineStr">
         <is>
-          <t>join-room.messages.invalid-team</t>
+          <t>join-room.messages.invalid-room-id</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>Field 'team' must be 'red', 'black', null, or undefined</t>
+          <t>Field 'id' is required and must be a positive integer</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>Trường 'team' phải là 'red', 'black', null hoặc không truyền</t>
+          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
         </is>
       </c>
     </row>
     <row r="223" ht="18" customHeight="1">
       <c r="A223" s="1" t="inlineStr">
         <is>
-          <t>join-room.messages.invalid-room-id</t>
+          <t>join-room.messages.room-not-found</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
         <is>
-          <t>Field 'id' is required and must be a positive integer</t>
+          <t>Room not found</t>
         </is>
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
+          <t>Không tìm thấy phòng</t>
         </is>
       </c>
     </row>
     <row r="224" ht="18" customHeight="1">
       <c r="A224" s="1" t="inlineStr">
         <is>
-          <t>join-room.messages.room-not-found</t>
+          <t>join-room.messages.success</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t>Room not found</t>
+          <t>Successfully joined the room</t>
         </is>
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy phòng</t>
+          <t>Tham gia phòng thành công</t>
         </is>
       </c>
     </row>
     <row r="225" ht="18" customHeight="1">
       <c r="A225" s="1" t="inlineStr">
         <is>
-          <t>join-room.messages.success</t>
+          <t>join-room.messages.team-seat-occupied</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t>Successfully joined the room</t>
+          <t>Selected team seat is already occupied</t>
         </is>
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>Tham gia phòng thành công</t>
+          <t>Vị trí đội đã chọn đã có người chơi</t>
         </is>
       </c>
     </row>
     <row r="226" ht="18" customHeight="1">
       <c r="A226" s="1" t="inlineStr">
         <is>
-          <t>join-room.messages.team-seat-occupied</t>
+          <t>kick-user.messages.cannot-kick-self</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
         <is>
-          <t>Selected team seat is already occupied</t>
+          <t>You cannot kick yourself</t>
         </is>
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>Vị trí đội đã chọn đã có người chơi</t>
+          <t>Bạn không thể kick chính mình</t>
         </is>
       </c>
     </row>
     <row r="227" ht="18" customHeight="1">
       <c r="A227" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.cannot-kick-self</t>
+          <t>kick-user.messages.forbidden</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
         <is>
-          <t>You cannot kick yourself</t>
+          <t>Only the host can kick users</t>
         </is>
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>Bạn không thể kick chính mình</t>
+          <t>Chỉ chủ phòng mới có thể kick người dùng</t>
         </is>
       </c>
     </row>
     <row r="228" ht="18" customHeight="1">
       <c r="A228" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.forbidden</t>
+          <t>kick-user.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>Only the host can kick users</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>Chỉ chủ phòng mới có thể kick người dùng</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="229" ht="18" customHeight="1">
       <c r="A229" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.internal-server-error</t>
+          <t>kick-user.messages.invalid-room-id</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Field 'id' is required and must be a positive integer</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
         </is>
       </c>
     </row>
     <row r="230" ht="18" customHeight="1">
       <c r="A230" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.invalid-room-id</t>
+          <t>kick-user.messages.invalid-user-id</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>Field 'id' is required and must be a positive integer</t>
+          <t>Field 'userId' is required and must be a positive integer</t>
         </is>
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
+          <t>Trường 'userId' là bắt buộc và phải là số nguyên dương</t>
         </is>
       </c>
     </row>
     <row r="231" ht="18" customHeight="1">
       <c r="A231" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.invalid-user-id</t>
+          <t>kick-user.messages.room-not-found</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t>Field 'userId' is required and must be a positive integer</t>
+          <t>Room not found</t>
         </is>
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>Trường 'userId' là bắt buộc và phải là số nguyên dương</t>
+          <t>Không tìm thấy phòng</t>
         </is>
       </c>
     </row>
     <row r="232" ht="18" customHeight="1">
       <c r="A232" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.room-not-found</t>
+          <t>kick-user.messages.room-not-waiting</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
         <is>
-          <t>Room not found</t>
+          <t>You can only kick users while the room is waiting</t>
         </is>
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy phòng</t>
+          <t>Chỉ có thể kick người dùng khi phòng đang ở trạng thái chờ</t>
         </is>
       </c>
     </row>
     <row r="233" ht="18" customHeight="1">
       <c r="A233" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.room-not-waiting</t>
+          <t>kick-user.messages.success</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
         <is>
-          <t>You can only kick users while the room is waiting</t>
+          <t>User has been kicked</t>
         </is>
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>Chỉ có thể kick người dùng khi phòng đang ở trạng thái chờ</t>
+          <t>Người dùng đã bị kick</t>
         </is>
       </c>
     </row>
     <row r="234" ht="18" customHeight="1">
       <c r="A234" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.success</t>
+          <t>kick-user.messages.user-not-in-room</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>User has been kicked</t>
+          <t>User is not in this room</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>Người dùng đã bị kick</t>
+          <t>Người dùng không trong phòng này</t>
         </is>
       </c>
     </row>
     <row r="235" ht="18" customHeight="1">
       <c r="A235" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.user-not-in-room</t>
+          <t>kick-user.messages.you-were-kicked</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
         <is>
-          <t>User is not in this room</t>
+          <t>You have been removed from the room by the host</t>
         </is>
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>Người dùng không trong phòng này</t>
+          <t>Bạn đã bị chủ phòng đưa ra khỏi phòng</t>
         </is>
       </c>
     </row>
     <row r="236" ht="18" customHeight="1">
       <c r="A236" s="1" t="inlineStr">
         <is>
-          <t>kick-user.messages.you-were-kicked</t>
+          <t>leave-room.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>You have been removed from the room by the host</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>Bạn đã bị chủ phòng đưa ra khỏi phòng</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="237" ht="18" customHeight="1">
       <c r="A237" s="1" t="inlineStr">
         <is>
-          <t>leave-room.messages.internal-server-error</t>
+          <t>leave-room.messages.invalid-room-id</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Field 'id' is required and must be a positive integer</t>
         </is>
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
         </is>
       </c>
     </row>
     <row r="238" ht="18" customHeight="1">
       <c r="A238" s="1" t="inlineStr">
         <is>
-          <t>leave-room.messages.invalid-room-id</t>
+          <t>leave-room.messages.player-not-in-room</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>Field 'id' is required and must be a positive integer</t>
+          <t>Player is not in this room</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
+          <t>Người chơi không trong phòng này</t>
         </is>
       </c>
     </row>
     <row r="239" ht="18" customHeight="1">
       <c r="A239" s="1" t="inlineStr">
         <is>
-          <t>leave-room.messages.player-not-in-room</t>
+          <t>leave-room.messages.success</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
         <is>
-          <t>Player is not in this room</t>
+          <t>Leave room successfully</t>
         </is>
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>Người chơi không trong phòng này</t>
+          <t>Rời phòng thành công</t>
         </is>
       </c>
     </row>
     <row r="240" ht="18" customHeight="1">
       <c r="A240" s="1" t="inlineStr">
         <is>
-          <t>leave-room.messages.success</t>
+          <t>load-room.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
         <is>
-          <t>Leave room successfully</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>Rời phòng thành công</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="241" ht="18" customHeight="1">
       <c r="A241" s="1" t="inlineStr">
         <is>
-          <t>load-room.messages.internal-server-error</t>
+          <t>load-room.messages.invalid-room-id</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Room ID must be a positive integer</t>
         </is>
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>ID phòng phải là số nguyên dương</t>
         </is>
       </c>
     </row>
     <row r="242" ht="18" customHeight="1">
       <c r="A242" s="1" t="inlineStr">
         <is>
-          <t>load-room.messages.invalid-room-id</t>
+          <t>load-room.messages.room-not-found</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>Room ID must be a positive integer</t>
+          <t>Room not found</t>
         </is>
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>ID phòng phải là số nguyên dương</t>
+          <t>Không tìm thấy phòng</t>
         </is>
       </c>
     </row>
     <row r="243" ht="18" customHeight="1">
       <c r="A243" s="1" t="inlineStr">
         <is>
-          <t>load-room.messages.room-not-found</t>
+          <t>load-room.messages.success</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>Room not found</t>
+          <t>Load room successfully</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy phòng</t>
+          <t>Tải phòng thành công</t>
         </is>
       </c>
     </row>
     <row r="244" ht="18" customHeight="1">
       <c r="A244" s="1" t="inlineStr">
         <is>
-          <t>load-room.messages.success</t>
+          <t>google-login.messages.email-not-verified</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>Load room successfully</t>
+          <t>Your Google email is not verified</t>
         </is>
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>Tải phòng thành công</t>
+          <t>Email Google của bạn chưa được xác minh</t>
         </is>
       </c>
     </row>
     <row r="245" ht="18" customHeight="1">
       <c r="A245" s="1" t="inlineStr">
         <is>
-          <t>google-login.messages.email-not-verified</t>
+          <t>google-login.messages.failed</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
         <is>
-          <t>Your Google email is not verified</t>
+          <t>Login failed</t>
         </is>
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>Email Google của bạn chưa được xác minh</t>
+          <t>Đăng nhập không thành công</t>
         </is>
       </c>
     </row>
     <row r="246" ht="18" customHeight="1">
       <c r="A246" s="1" t="inlineStr">
         <is>
-          <t>google-login.messages.failed</t>
+          <t>google-login.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
         <is>
-          <t>Login failed</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>Đăng nhập không thành công</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="247" ht="18" customHeight="1">
       <c r="A247" s="1" t="inlineStr">
         <is>
-          <t>google-login.messages.internal-server-error</t>
+          <t>google-login.messages.invalid-token</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Invalid Google credential</t>
         </is>
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Thông tin đăng nhập Google không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="248" ht="18" customHeight="1">
       <c r="A248" s="1" t="inlineStr">
         <is>
-          <t>google-login.messages.invalid-token</t>
+          <t>google-login.messages.missing-credential</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>Invalid Google credential</t>
+          <t>Google credential is required</t>
         </is>
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>Thông tin đăng nhập Google không hợp lệ</t>
+          <t>Thiếu thông tin đăng nhập Google</t>
         </is>
       </c>
     </row>
     <row r="249" ht="18" customHeight="1">
       <c r="A249" s="1" t="inlineStr">
         <is>
-          <t>google-login.messages.missing-credential</t>
+          <t>facebook-login.messages.missing-token</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
         <is>
-          <t>Google credential is required</t>
+          <t>Facebook token is required</t>
         </is>
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>Thiếu thông tin đăng nhập Google</t>
+          <t>Thiếu thông tin đăng nhập Facebook</t>
         </is>
       </c>
     </row>
     <row r="250" ht="18" customHeight="1">
       <c r="A250" s="1" t="inlineStr">
         <is>
-          <t>facebook-login.messages.missing-token</t>
+          <t>facebook-login.messages.invalid-token</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>Facebook token is required</t>
+          <t>Invalid Facebook token</t>
         </is>
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>Thiếu thông tin đăng nhập Facebook</t>
+          <t>Thông tin đăng nhập Facebook không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="251" ht="18" customHeight="1">
       <c r="A251" s="1" t="inlineStr">
         <is>
-          <t>facebook-login.messages.invalid-token</t>
+          <t>facebook-login.messages.not-linked</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>Invalid Facebook token</t>
+          <t>This Facebook account is not linked. Log in another way and link it in Settings</t>
         </is>
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>Thông tin đăng nhập Facebook không hợp lệ</t>
+          <t>Tài khoản Facebook này chưa được liên kết. Hãy đăng nhập cách khác rồi liên kết trong Cài đặt</t>
         </is>
       </c>
     </row>
     <row r="252" ht="18" customHeight="1">
       <c r="A252" s="1" t="inlineStr">
         <is>
-          <t>facebook-login.messages.not-linked</t>
+          <t>facebook-login.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B252" s="2" t="inlineStr">
         <is>
-          <t>This Facebook account is not linked. Log in another way and link it in Settings</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản Facebook này chưa được liên kết. Hãy đăng nhập cách khác rồi liên kết trong Cài đặt</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="253" ht="18" customHeight="1">
       <c r="A253" s="1" t="inlineStr">
         <is>
-          <t>facebook-login.messages.internal-server-error</t>
+          <t>facebook-link.messages.missing-token</t>
         </is>
       </c>
       <c r="B253" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Facebook token is required</t>
         </is>
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Thiếu thông tin đăng nhập Facebook</t>
         </is>
       </c>
     </row>
     <row r="254" ht="18" customHeight="1">
       <c r="A254" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.missing-token</t>
+          <t>facebook-link.messages.invalid-token</t>
         </is>
       </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
-          <t>Facebook token is required</t>
+          <t>Invalid Facebook token</t>
         </is>
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>Thiếu thông tin đăng nhập Facebook</t>
+          <t>Thông tin đăng nhập Facebook không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="255" ht="18" customHeight="1">
       <c r="A255" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.invalid-token</t>
+          <t>facebook-link.messages.linked</t>
         </is>
       </c>
       <c r="B255" s="2" t="inlineStr">
         <is>
-          <t>Invalid Facebook token</t>
+          <t>Facebook linked successfully</t>
         </is>
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>Thông tin đăng nhập Facebook không hợp lệ</t>
+          <t>Đã liên kết Facebook</t>
         </is>
       </c>
     </row>
     <row r="256" ht="18" customHeight="1">
       <c r="A256" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.linked</t>
+          <t>facebook-link.messages.already-linked</t>
         </is>
       </c>
       <c r="B256" s="2" t="inlineStr">
         <is>
-          <t>Facebook linked successfully</t>
+          <t>This Facebook account is already linked to your account</t>
         </is>
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>Đã liên kết Facebook</t>
+          <t>Tài khoản Facebook này đã được liên kết với bạn</t>
         </is>
       </c>
     </row>
     <row r="257" ht="18" customHeight="1">
       <c r="A257" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.already-linked</t>
+          <t>facebook-link.messages.linked-to-other</t>
         </is>
       </c>
       <c r="B257" s="2" t="inlineStr">
         <is>
-          <t>This Facebook account is already linked to your account</t>
+          <t>This Facebook account is already linked to another account</t>
         </is>
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản Facebook này đã được liên kết với bạn</t>
+          <t>Tài khoản Facebook này đã được liên kết với tài khoản khác</t>
         </is>
       </c>
     </row>
     <row r="258" ht="18" customHeight="1">
       <c r="A258" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.linked-to-other</t>
+          <t>facebook-link.messages.already-has-facebook</t>
         </is>
       </c>
       <c r="B258" s="2" t="inlineStr">
         <is>
-          <t>This Facebook account is already linked to another account</t>
+          <t>You already linked a different Facebook account</t>
         </is>
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>Tài khoản Facebook này đã được liên kết với tài khoản khác</t>
+          <t>Bạn đã liên kết một tài khoản Facebook khác</t>
         </is>
       </c>
     </row>
     <row r="259" ht="18" customHeight="1">
       <c r="A259" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.already-has-facebook</t>
+          <t>facebook-link.messages.unlinked</t>
         </is>
       </c>
       <c r="B259" s="2" t="inlineStr">
         <is>
-          <t>You already linked a different Facebook account</t>
+          <t>Facebook unlinked</t>
         </is>
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>Bạn đã liên kết một tài khoản Facebook khác</t>
+          <t>Đã huỷ liên kết Facebook</t>
         </is>
       </c>
     </row>
     <row r="260" ht="36" customHeight="1">
       <c r="A260" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.unlinked</t>
+          <t>facebook-link.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B260" s="2" t="inlineStr">
         <is>
-          <t>Facebook unlinked</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>Đã huỷ liên kết Facebook</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="261" ht="36" customHeight="1">
       <c r="A261" s="1" t="inlineStr">
         <is>
-          <t>facebook-link.messages.internal-server-error</t>
+          <t>logout.messages.already-inactive</t>
         </is>
       </c>
       <c r="B261" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Session already inactive</t>
         </is>
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Phiên đã ngưng hoạt động</t>
         </is>
       </c>
     </row>
     <row r="262" ht="18" customHeight="1">
       <c r="A262" s="1" t="inlineStr">
         <is>
-          <t>logout.messages.already-inactive</t>
+          <t>logout.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B262" s="2" t="inlineStr">
         <is>
-          <t>Session already inactive</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>Phiên đã ngưng hoạt động</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="263" ht="18" customHeight="1">
       <c r="A263" s="1" t="inlineStr">
         <is>
-          <t>logout.messages.internal-server-error</t>
+          <t>logout.messages.success</t>
         </is>
       </c>
       <c r="B263" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Logout successful</t>
         </is>
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Đăng xuất thành công</t>
         </is>
       </c>
     </row>
     <row r="264" ht="18" customHeight="1">
       <c r="A264" s="1" t="inlineStr">
         <is>
-          <t>logout.messages.success</t>
+          <t>refresh-token.messages.missing-refresh-token</t>
         </is>
       </c>
       <c r="B264" s="2" t="inlineStr">
         <is>
-          <t>Logout successful</t>
+          <t>Missing refresh token cookie</t>
         </is>
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>Đăng xuất thành công</t>
+          <t>Thiếu cookie token làm mới</t>
         </is>
       </c>
     </row>
     <row r="265" ht="17" customHeight="1">
       <c r="A265" s="1" t="inlineStr">
         <is>
-          <t>refresh-token.messages.missing-refresh-token</t>
+          <t>refresh-token.messages.mismatch-or-expired</t>
         </is>
       </c>
       <c r="B265" s="1" t="inlineStr">
         <is>
-          <t>Missing refresh token cookie</t>
+          <t>Refresh token mismatch or expired</t>
         </is>
       </c>
       <c r="C265" s="1" t="inlineStr">
         <is>
-          <t>Thiếu cookie token làm mới</t>
+          <t>Thiếu refresh token hoặc đã hết hạn</t>
         </is>
       </c>
     </row>
     <row r="266" ht="18" customHeight="1">
       <c r="A266" s="2" t="inlineStr">
         <is>
-          <t>refresh-token.messages.mismatch-or-expired</t>
+          <t>refresh-token.messages.success</t>
         </is>
       </c>
       <c r="B266" s="2" t="inlineStr">
         <is>
-          <t>Refresh token mismatch or expired</t>
+          <t>Token refreshed</t>
         </is>
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>Thiếu refresh token hoặc đã hết hạn</t>
+          <t>Token đã làm mới</t>
         </is>
       </c>
     </row>
     <row r="267" ht="18" customHeight="1">
       <c r="A267" s="2" t="inlineStr">
         <is>
-          <t>refresh-token.messages.success</t>
+          <t>register.messages.email-exists</t>
         </is>
       </c>
       <c r="B267" s="2" t="inlineStr">
         <is>
-          <t>Token refreshed</t>
+          <t>Email already exists</t>
         </is>
       </c>
       <c r="C267" s="2" t="inlineStr">
         <is>
-          <t>Token đã làm mới</t>
+          <t>Email đã tồn tại</t>
         </is>
       </c>
     </row>
     <row r="268" ht="18" customHeight="1">
       <c r="A268" s="2" t="inlineStr">
         <is>
-          <t>register.messages.email-exists</t>
+          <t>register.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B268" s="2" t="inlineStr">
         <is>
-          <t>Email already exists</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>Email đã tồn tại</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="269" ht="18" customHeight="1">
       <c r="A269" s="2" t="inlineStr">
         <is>
-          <t>register.messages.internal-server-error</t>
+          <t>register.messages.missing-fields</t>
         </is>
       </c>
       <c r="B269" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Username, password, gender, displayName and email are required</t>
         </is>
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Tên người dùng, mật khẩu, giới tính, tên hiển thị và email là bắt buộc</t>
         </is>
       </c>
     </row>
     <row r="270" ht="18" customHeight="1">
       <c r="A270" s="2" t="inlineStr">
         <is>
-          <t>register.messages.missing-fields</t>
+          <t>register.messages.success</t>
         </is>
       </c>
       <c r="B270" s="2" t="inlineStr">
         <is>
-          <t>Username, password, gender, displayName and email are required</t>
+          <t>User created successfully</t>
         </is>
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>Tên người dùng, mật khẩu, giới tính, tên hiển thị và email là bắt buộc</t>
+          <t>Người dùng được tạo thành công</t>
         </is>
       </c>
     </row>
     <row r="271" ht="36" customHeight="1">
       <c r="A271" s="2" t="inlineStr">
         <is>
-          <t>register.messages.success</t>
+          <t>register.messages.username-exists</t>
         </is>
       </c>
       <c r="B271" s="2" t="inlineStr">
         <is>
-          <t>User created successfully</t>
+          <t>Username already exists</t>
         </is>
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>Người dùng được tạo thành công</t>
+          <t>Tên người dùng đã tồn tại</t>
         </is>
       </c>
     </row>
     <row r="272" ht="36" customHeight="1">
       <c r="A272" s="2" t="inlineStr">
         <is>
-          <t>register.messages.username-exists</t>
+          <t>reset-password.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B272" s="2" t="inlineStr">
         <is>
-          <t>Username already exists</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>Tên người dùng đã tồn tại</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="273" ht="18" customHeight="1">
       <c r="A273" s="2" t="inlineStr">
         <is>
-          <t>reset-password.messages.internal-server-error</t>
+          <t>reset-password.messages.invalid-or-expired-token</t>
         </is>
       </c>
       <c r="B273" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Invalid or expired reset password token</t>
         </is>
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Token đặt lại mật khẩu không hợp lệ hoặc đã hết hạn</t>
         </is>
       </c>
     </row>
     <row r="274" ht="18" customHeight="1">
       <c r="A274" s="1" t="inlineStr">
         <is>
-          <t>reset-password.messages.invalid-or-expired-token</t>
+          <t>reset-password.messages.invalid-user-id</t>
         </is>
       </c>
       <c r="B274" s="2" t="inlineStr">
         <is>
-          <t>Invalid or expired reset password token</t>
+          <t>Invalid user id</t>
         </is>
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>Token đặt lại mật khẩu không hợp lệ hoặc đã hết hạn</t>
+          <t>ID người dùng không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="275" ht="18" customHeight="1">
       <c r="A275" s="1" t="inlineStr">
         <is>
-          <t>reset-password.messages.invalid-user-id</t>
+          <t>reset-password.messages.missing-id-or-token</t>
         </is>
       </c>
       <c r="B275" s="2" t="inlineStr">
         <is>
-          <t>Invalid user id</t>
+          <t>ID and token are required</t>
         </is>
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>ID người dùng không hợp lệ</t>
+          <t>ID và token là bắt buộc</t>
         </is>
       </c>
     </row>
     <row r="276" ht="18" customHeight="1">
       <c r="A276" s="1" t="inlineStr">
         <is>
-          <t>reset-password.messages.missing-id-or-token</t>
+          <t>reset-password.messages.missing-userId-or-password</t>
         </is>
       </c>
       <c r="B276" s="2" t="inlineStr">
         <is>
-          <t>ID and token are required</t>
+          <t>UserId and password are required</t>
         </is>
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>ID và token là bắt buộc</t>
+          <t>UserId và mật khẩu là bắt buộc</t>
         </is>
       </c>
     </row>
     <row r="277" ht="18" customHeight="1">
       <c r="A277" s="1" t="inlineStr">
         <is>
-          <t>reset-password.messages.missing-userId-or-password</t>
+          <t>reset-password.messages.token-valid</t>
         </is>
       </c>
       <c r="B277" s="2" t="inlineStr">
         <is>
-          <t>UserId and password are required</t>
+          <t>Reset password token is valid</t>
         </is>
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>UserId và mật khẩu là bắt buộc</t>
+          <t>Token đặt lại mật khẩu hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="278" ht="18" customHeight="1">
       <c r="A278" s="1" t="inlineStr">
         <is>
-          <t>reset-password.messages.token-valid</t>
+          <t>reset-password.messages.user-not-found</t>
         </is>
       </c>
       <c r="B278" s="2" t="inlineStr">
         <is>
-          <t>Reset password token is valid</t>
+          <t>User not found</t>
         </is>
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>Token đặt lại mật khẩu hợp lệ</t>
+          <t>Không tìm thấy người dùng</t>
         </is>
       </c>
     </row>
     <row r="279" ht="18" customHeight="1">
       <c r="A279" s="1" t="inlineStr">
         <is>
-          <t>reset-password.messages.user-not-found</t>
+          <t>room.actions.start-room</t>
         </is>
       </c>
       <c r="B279" s="2" t="inlineStr">
         <is>
-          <t>User not found</t>
+          <t>Start room</t>
         </is>
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy người dùng</t>
+          <t>Bắt đầu chơi</t>
         </is>
       </c>
     </row>
     <row r="280" ht="18" customHeight="1">
       <c r="A280" s="1" t="inlineStr">
         <is>
-          <t>room.actions.start-room</t>
+          <t>room.actions.challenge</t>
         </is>
       </c>
       <c r="B280" s="2" t="inlineStr">
         <is>
-          <t>Start room</t>
+          <t>Challenge</t>
         </is>
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>Bắt đầu chơi</t>
+          <t>Vào chơi</t>
         </is>
       </c>
     </row>
     <row r="281" ht="18" customHeight="1">
       <c r="A281" s="1" t="inlineStr">
         <is>
-          <t>room.actions.challenge</t>
+          <t>room.actions.leave-seat</t>
         </is>
       </c>
       <c r="B281" s="2" t="inlineStr">
         <is>
-          <t>Challenge</t>
+          <t>Leave seat</t>
         </is>
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>Vào chơi</t>
+          <t>Ra xem</t>
         </is>
       </c>
     </row>
     <row r="282" ht="18" customHeight="1">
       <c r="A282" s="1" t="inlineStr">
         <is>
-          <t>room.actions.leave-seat</t>
+          <t>room.actions.undo</t>
         </is>
       </c>
       <c r="B282" s="2" t="inlineStr">
         <is>
-          <t>Leave seat</t>
+          <t>Undo</t>
         </is>
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>Ra xem</t>
+          <t>Hoán tác</t>
         </is>
       </c>
     </row>
     <row r="283" ht="18" customHeight="1">
       <c r="A283" s="1" t="inlineStr">
         <is>
-          <t>room.actions.undo</t>
+          <t>room.actions.surrender</t>
         </is>
       </c>
       <c r="B283" s="2" t="inlineStr">
         <is>
-          <t>Undo</t>
+          <t>Surrender</t>
         </is>
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>Hoán tác</t>
+          <t>Đầu hàng</t>
         </is>
       </c>
     </row>
     <row r="284" ht="18" customHeight="1">
       <c r="A284" s="1" t="inlineStr">
         <is>
-          <t>room.actions.surrender</t>
+          <t>room.actions.draw</t>
         </is>
       </c>
       <c r="B284" s="2" t="inlineStr">
         <is>
-          <t>Surrender</t>
+          <t>Draw</t>
         </is>
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>Đầu hàng</t>
+          <t>Hòa</t>
         </is>
       </c>
     </row>
     <row r="285" ht="18" customHeight="1">
       <c r="A285" s="1" t="inlineStr">
         <is>
-          <t>room.actions.draw</t>
+          <t>room.actions.back-home</t>
         </is>
       </c>
       <c r="B285" s="2" t="inlineStr">
         <is>
-          <t>Draw</t>
+          <t>Back to home</t>
         </is>
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>Hòa</t>
+          <t>Thoát phòng</t>
         </is>
       </c>
     </row>
     <row r="286" ht="18" customHeight="1">
       <c r="A286" s="1" t="inlineStr">
         <is>
-          <t>room.actions.back-home</t>
+          <t>room.actions.flip-board</t>
         </is>
       </c>
       <c r="B286" s="2" t="inlineStr">
         <is>
-          <t>Back to home</t>
+          <t>Flip board</t>
         </is>
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>Thoát phòng</t>
+          <t>Đảo chiều bàn cờ</t>
         </is>
       </c>
     </row>
     <row r="287" ht="18" customHeight="1">
       <c r="A287" s="1" t="inlineStr">
         <is>
-          <t>room.actions.flip-board</t>
+          <t>room.actions.accept-draw</t>
         </is>
       </c>
       <c r="B287" s="2" t="inlineStr">
         <is>
-          <t>Flip board</t>
+          <t>Accept</t>
         </is>
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>Đảo chiều bàn cờ</t>
+          <t>Chấp nhận</t>
         </is>
       </c>
     </row>
     <row r="288" ht="18" customHeight="1">
       <c r="A288" s="1" t="inlineStr">
         <is>
-          <t>room.actions.accept-draw</t>
+          <t>room.actions.reject-draw</t>
         </is>
       </c>
       <c r="B288" s="2" t="inlineStr">
         <is>
-          <t>Accept</t>
+          <t>Reject</t>
         </is>
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>Chấp nhận</t>
+          <t>Từ chối</t>
         </is>
       </c>
     </row>
     <row r="289" ht="18" customHeight="1">
       <c r="A289" s="1" t="inlineStr">
         <is>
-          <t>room.actions.reject-draw</t>
+          <t>room.actions.send-pm</t>
         </is>
       </c>
       <c r="B289" s="2" t="inlineStr">
         <is>
-          <t>Reject</t>
+          <t>Send PM</t>
         </is>
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>Từ chối</t>
+          <t>Chat</t>
         </is>
       </c>
     </row>
     <row r="290" ht="18" customHeight="1">
       <c r="A290" s="1" t="inlineStr">
         <is>
-          <t>room.actions.send-pm</t>
+          <t>room.actions.view-history</t>
         </is>
       </c>
       <c r="B290" s="2" t="inlineStr">
         <is>
-          <t>Send PM</t>
+          <t>History</t>
         </is>
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Lịch sử</t>
         </is>
       </c>
     </row>
     <row r="291" ht="18" customHeight="1">
       <c r="A291" s="1" t="inlineStr">
         <is>
-          <t>room.actions.view-history</t>
+          <t>room.actions.kick</t>
         </is>
       </c>
       <c r="B291" s="2" t="inlineStr">
         <is>
-          <t>History</t>
+          <t>Kick</t>
         </is>
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>Lịch sử</t>
+          <t>Kick</t>
         </is>
       </c>
     </row>
     <row r="292" ht="18" customHeight="1">
       <c r="A292" s="1" t="inlineStr">
         <is>
-          <t>room.actions.kick</t>
+          <t>room.actions.back-to-room</t>
         </is>
       </c>
       <c r="B292" s="2" t="inlineStr">
         <is>
-          <t>Kick</t>
+          <t>Back to room</t>
         </is>
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>Kick</t>
+          <t>Quay lại phòng chơi</t>
         </is>
       </c>
     </row>
     <row r="293" ht="18" customHeight="1">
       <c r="A293" s="1" t="inlineStr">
         <is>
-          <t>room.actions.back-to-room</t>
+          <t>room.actions.chat</t>
         </is>
       </c>
       <c r="B293" s="2" t="inlineStr">
         <is>
-          <t>Back to room</t>
+          <t>Room chat</t>
         </is>
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>Quay lại phòng chơi</t>
+          <t>Phòng chat</t>
         </is>
       </c>
     </row>
     <row r="294" ht="18" customHeight="1">
       <c r="A294" s="1" t="inlineStr">
         <is>
-          <t>room.actions.chat</t>
+          <t>room.messages.draw-accepted</t>
         </is>
       </c>
       <c r="B294" s="2" t="inlineStr">
         <is>
-          <t>Room chat</t>
+          <t>Opponent accepted the draw</t>
         </is>
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>Phòng chat</t>
+          <t>Đối phương đã đồng ý hòa</t>
         </is>
       </c>
     </row>
     <row r="295" ht="18" customHeight="1">
       <c r="A295" s="1" t="inlineStr">
         <is>
-          <t>room.messages.draw-accepted</t>
+          <t>room.messages.draw-rejected</t>
         </is>
       </c>
       <c r="B295" s="2" t="inlineStr">
         <is>
-          <t>Opponent accepted the draw</t>
+          <t>Opponent rejected the draw</t>
         </is>
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>Đối phương đã đồng ý hòa</t>
+          <t>Đối phương từ chối hòa</t>
         </is>
       </c>
     </row>
     <row r="296" ht="18" customHeight="1">
       <c r="A296" s="1" t="inlineStr">
         <is>
-          <t>room.messages.draw-rejected</t>
+          <t>room.messages.opponent-surrendered</t>
         </is>
       </c>
       <c r="B296" s="2" t="inlineStr">
         <is>
-          <t>Opponent rejected the draw</t>
+          <t>Opponent surrendered! You won!</t>
         </is>
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>Đối phương từ chối hòa</t>
+          <t>Đối phương đã đầu hàng! Bạn thắng!</t>
         </is>
       </c>
     </row>
     <row r="297" ht="18" customHeight="1">
       <c r="A297" s="1" t="inlineStr">
         <is>
-          <t>room.messages.opponent-surrendered</t>
+          <t>room.messages.confirm-leave</t>
         </is>
       </c>
       <c r="B297" s="2" t="inlineStr">
         <is>
-          <t>Opponent surrendered! You won!</t>
+          <t>Are you sure you want to leave room?</t>
         </is>
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>Đối phương đã đầu hàng! Bạn thắng!</t>
+          <t>Bạn có chắc muốn rời bàn chơi?</t>
         </is>
       </c>
     </row>
     <row r="298" ht="18" customHeight="1">
       <c r="A298" s="1" t="inlineStr">
         <is>
-          <t>room.messages.confirm-leave</t>
+          <t>room.messages.confirm-surrender</t>
         </is>
       </c>
       <c r="B298" s="2" t="inlineStr">
         <is>
-          <t>Are you sure you want to leave room?</t>
+          <t>Are you sure you want to surrender?</t>
         </is>
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>Bạn có chắc muốn rời bàn chơi?</t>
+          <t>Bạn có chắc chắn muốn đầu hàng không?</t>
         </is>
       </c>
     </row>
     <row r="299" ht="18" customHeight="1">
       <c r="A299" s="1" t="inlineStr">
         <is>
-          <t>room.messages.confirm-surrender</t>
+          <t>room.messages.confirm-draw</t>
         </is>
       </c>
       <c r="B299" s="2" t="inlineStr">
         <is>
-          <t>Are you sure you want to surrender?</t>
+          <t>Are you sure you want to draw?</t>
         </is>
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>Bạn có chắc chắn muốn đầu hàng không?</t>
+          <t>Bạn có chắc chắn muốn hòa không?</t>
         </is>
       </c>
     </row>
     <row r="300" ht="18" customHeight="1">
       <c r="A300" s="1" t="inlineStr">
         <is>
-          <t>room.messages.confirm-draw</t>
+          <t>room.messages.confirm-accept-draw</t>
         </is>
       </c>
       <c r="B300" s="2" t="inlineStr">
         <is>
-          <t>Are you sure you want to draw?</t>
+          <t>Opponent has proposed a draw. Do you accept?</t>
         </is>
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>Bạn có chắc chắn muốn hòa không?</t>
+          <t>Đối phương đã chủ hòa, bạn có đồng ý không?</t>
         </is>
       </c>
     </row>
     <row r="301" ht="18" customHeight="1">
       <c r="A301" s="1" t="inlineStr">
         <is>
-          <t>room.messages.confirm-accept-draw</t>
+          <t>room.messages.insufficient-amount</t>
         </is>
       </c>
       <c r="B301" s="2" t="inlineStr">
         <is>
-          <t>Opponent has proposed a draw. Do you accept?</t>
+          <t>You do not have enough balance to join this room</t>
         </is>
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>Đối phương đã chủ hòa, bạn có đồng ý không?</t>
+          <t>Bạn không đủ tiền để tham gia bàn chơi này</t>
         </is>
       </c>
     </row>
     <row r="302" ht="18" customHeight="1">
       <c r="A302" s="1" t="inlineStr">
         <is>
-          <t>room.messages.insufficient-amount</t>
+          <t>room.messages.will-leave-current-room</t>
         </is>
       </c>
       <c r="B302" s="2" t="inlineStr">
         <is>
-          <t>You do not have enough balance to join this room</t>
+          <t>You are currently in another room. Joining this room will remove you from the current room</t>
         </is>
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>Bạn không đủ tiền để tham gia bàn chơi này</t>
+          <t>Bạn đang ở trong một phòng khác. Tham gia phòng này sẽ loại bạn ra khỏi phòng hiện tại</t>
         </is>
       </c>
     </row>
     <row r="303" ht="18" customHeight="1">
       <c r="A303" s="1" t="inlineStr">
         <is>
-          <t>room.messages.will-leave-current-room</t>
+          <t>room.messages.game-ended</t>
         </is>
       </c>
       <c r="B303" s="2" t="inlineStr">
         <is>
-          <t>You are currently in another room. Joining this room will remove you from the current room</t>
+          <t>Game ended</t>
         </is>
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>Bạn đang ở trong một phòng khác. Tham gia phòng này sẽ loại bạn ra khỏi phòng hiện tại</t>
+          <t>Ván đấu đã kết thúc</t>
         </is>
       </c>
     </row>
     <row r="304" ht="18" customHeight="1">
       <c r="A304" s="1" t="inlineStr">
         <is>
-          <t>room.messages.game-ended</t>
+          <t>room.messages.you-win</t>
         </is>
       </c>
       <c r="B304" s="2" t="inlineStr">
         <is>
-          <t>Game ended</t>
+          <t>You win</t>
         </is>
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>Ván đấu đã kết thúc</t>
+          <t>Bạn đã chiến thắng</t>
         </is>
       </c>
     </row>
     <row r="305" ht="18" customHeight="1">
       <c r="A305" s="1" t="inlineStr">
         <is>
-          <t>room.messages.you-win</t>
+          <t>room.messages.you-lose</t>
         </is>
       </c>
       <c r="B305" s="2" t="inlineStr">
         <is>
-          <t>You win</t>
+          <t>You lose</t>
         </is>
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>Bạn đã chiến thắng</t>
+          <t>Bạn đã thua</t>
         </is>
       </c>
     </row>
     <row r="306" ht="90" customHeight="1">
       <c r="A306" s="1" t="inlineStr">
         <is>
-          <t>room.messages.you-lose</t>
+          <t>room.messages.you-draw</t>
         </is>
       </c>
       <c r="B306" s="2" t="inlineStr">
         <is>
-          <t>You lose</t>
+          <t>The game is a draw</t>
         </is>
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>Bạn đã thua</t>
+          <t>Ván đấu hòa</t>
         </is>
       </c>
     </row>
     <row r="307" ht="90" customHeight="1">
       <c r="A307" s="1" t="inlineStr">
         <is>
-          <t>room.messages.you-draw</t>
+          <t>room.messages.you-win-per-move-timeout</t>
         </is>
       </c>
       <c r="B307" s="2" t="inlineStr">
         <is>
-          <t>The game is a draw</t>
+          <t>You win — your opponent ran out of move time</t>
         </is>
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>Ván đấu hòa</t>
+          <t>Bạn thắng vì đối thủ hết giờ đi một nước</t>
         </is>
       </c>
     </row>
     <row r="308" ht="18" customHeight="1">
       <c r="A308" s="1" t="inlineStr">
         <is>
-          <t>room.messages.you-win-per-move-timeout</t>
+          <t>room.messages.you-lose-per-move-timeout</t>
         </is>
       </c>
       <c r="B308" s="2" t="inlineStr">
         <is>
-          <t>You win — your opponent ran out of move time</t>
+          <t>You lose — you ran out of move time</t>
         </is>
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>Bạn thắng vì đối thủ hết giờ đi một nước</t>
+          <t>Bạn thua do hết giờ đi một nước</t>
         </is>
       </c>
     </row>
     <row r="309" ht="18" customHeight="1">
       <c r="A309" s="1" t="inlineStr">
         <is>
-          <t>room.messages.you-lose-per-move-timeout</t>
+          <t>room.messages.spectator-win-checkmate</t>
         </is>
       </c>
       <c r="B309" s="2" t="inlineStr">
         <is>
-          <t>You lose — you ran out of move time</t>
+          <t>{0} won by checkmate</t>
         </is>
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>Bạn thua do hết giờ đi một nước</t>
+          <t>{0} thắng do chiếu bí</t>
         </is>
       </c>
     </row>
     <row r="310" ht="18" customHeight="1">
       <c r="A310" s="1" t="inlineStr">
         <is>
-          <t>room.messages.spectator-win-checkmate</t>
+          <t>room.messages.spectator-win-stalemate</t>
         </is>
       </c>
       <c r="B310" s="2" t="inlineStr">
         <is>
-          <t>{0} won by checkmate</t>
+          <t>{0} won — opponent had no legal moves</t>
         </is>
       </c>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>{0} thắng do chiếu bí</t>
+          <t>{0} thắng do đối thủ hết nước đi</t>
         </is>
       </c>
     </row>
     <row r="311" ht="18" customHeight="1">
       <c r="A311" s="2" t="inlineStr">
         <is>
-          <t>room.messages.spectator-win-stalemate</t>
+          <t>room.messages.spectator-win-timeout</t>
         </is>
       </c>
       <c r="B311" s="2" t="inlineStr">
         <is>
-          <t>{0} won — opponent had no legal moves</t>
+          <t>{0} won on time</t>
         </is>
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>{0} thắng do đối thủ hết nước đi</t>
+          <t>{0} thắng do đối thủ hết giờ</t>
         </is>
       </c>
     </row>
     <row r="312" ht="18" customHeight="1">
       <c r="A312" s="2" t="inlineStr">
         <is>
-          <t>room.messages.spectator-win-timeout</t>
+          <t>room.messages.spectator-win-per-move-timeout</t>
         </is>
       </c>
       <c r="B312" s="2" t="inlineStr">
         <is>
-          <t>{0} won on time</t>
+          <t>{0} won — opponent ran out of move time</t>
         </is>
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>{0} thắng do đối thủ hết giờ</t>
+          <t>{0} thắng do đối thủ hết giờ đi một nước</t>
         </is>
       </c>
     </row>
     <row r="313" ht="18" customHeight="1">
       <c r="A313" s="2" t="inlineStr">
         <is>
-          <t>room.messages.spectator-win-per-move-timeout</t>
+          <t>room.messages.spectator-draw</t>
         </is>
       </c>
       <c r="B313" s="2" t="inlineStr">
         <is>
-          <t>{0} won — opponent ran out of move time</t>
+          <t>The game ended in a draw</t>
         </is>
       </c>
       <c r="C313" s="2" t="inlineStr">
         <is>
-          <t>{0} thắng do đối thủ hết giờ đi một nước</t>
+          <t>Ván đấu kết thúc với tỉ số hòa</t>
         </is>
       </c>
     </row>
     <row r="314" ht="18" customHeight="1">
       <c r="A314" s="2" t="inlineStr">
         <is>
-          <t>room.messages.spectator-draw</t>
+          <t>room.messages.back-to-room</t>
         </is>
       </c>
       <c r="B314" s="2" t="inlineStr">
         <is>
-          <t>The game ended in a draw</t>
+          <t>Back to room</t>
         </is>
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>Ván đấu kết thúc với tỉ số hòa</t>
+          <t>Quay lại phòng</t>
         </is>
       </c>
     </row>
     <row r="315" ht="54" customHeight="1">
       <c r="A315" s="2" t="inlineStr">
         <is>
-          <t>room.messages.back-to-room</t>
+          <t>room.messages.auto-back-countdown</t>
         </is>
       </c>
       <c r="B315" s="2" t="inlineStr">
         <is>
-          <t>Back to room</t>
+          <t>{0}. Press the back button to return to the room. You will be automatically returned in {1}s</t>
         </is>
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>Quay lại phòng</t>
+          <t>{0}. Bấm nút quay lại để quay lại room. Bạn sẽ tự động quay lại trong {1}s</t>
         </is>
       </c>
     </row>
     <row r="316" ht="18" customHeight="1">
       <c r="A316" s="2" t="inlineStr">
         <is>
-          <t>room.messages.auto-back-countdown</t>
+          <t>room.notifications.joined</t>
         </is>
       </c>
       <c r="B316" s="2" t="inlineStr">
         <is>
-          <t>{0}. Press the back button to return to the room. You will be automatically returned in {1}s</t>
+          <t>{0} joined the room</t>
         </is>
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>{0}. Bấm nút quay lại để quay lại room. Bạn sẽ tự động quay lại trong {1}s</t>
+          <t>{0} đã vào phòng</t>
         </is>
       </c>
     </row>
     <row r="317" ht="90" customHeight="1">
       <c r="A317" s="2" t="inlineStr">
         <is>
-          <t>room.notifications.joined</t>
+          <t>room.notifications.left</t>
         </is>
       </c>
       <c r="B317" s="2" t="inlineStr">
         <is>
-          <t>{0} joined the room</t>
+          <t>{0} left the room</t>
         </is>
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>{0} đã vào phòng</t>
+          <t>{0} đã rời phòng</t>
         </is>
       </c>
     </row>
     <row r="318" ht="18" customHeight="1">
       <c r="A318" s="2" t="inlineStr">
         <is>
-          <t>room.notifications.left</t>
+          <t>room.settings.title</t>
         </is>
       </c>
       <c r="B318" s="2" t="inlineStr">
         <is>
-          <t>{0} left the room</t>
+          <t>Room Settings</t>
         </is>
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
-          <t>{0} đã rời phòng</t>
+          <t>Cài đặt phòng</t>
         </is>
       </c>
     </row>
     <row r="319" ht="36" customHeight="1">
       <c r="A319" s="2" t="inlineStr">
         <is>
-          <t>room.settings.title</t>
+          <t>room.settings.room-name</t>
         </is>
       </c>
       <c r="B319" s="2" t="inlineStr">
         <is>
-          <t>Room Settings</t>
+          <t>Room name</t>
         </is>
       </c>
       <c r="C319" s="2" t="inlineStr">
         <is>
-          <t>Cài đặt phòng</t>
+          <t>Tên phòng</t>
         </is>
       </c>
     </row>
     <row r="320" ht="18" customHeight="1">
       <c r="A320" s="2" t="inlineStr">
         <is>
-          <t>room.settings.room-name</t>
+          <t>room.settings.players</t>
         </is>
       </c>
       <c r="B320" s="2" t="inlineStr">
         <is>
-          <t>Room name</t>
+          <t>Spectators</t>
         </is>
       </c>
       <c r="C320" s="2" t="inlineStr">
         <is>
-          <t>Tên phòng</t>
+          <t>Người xem</t>
         </is>
       </c>
     </row>
     <row r="321" ht="72" customHeight="1">
       <c r="A321" s="2" t="inlineStr">
         <is>
-          <t>room.settings.players</t>
+          <t>room.settings.save</t>
         </is>
       </c>
       <c r="B321" s="2" t="inlineStr">
         <is>
-          <t>Spectators</t>
+          <t>Save</t>
         </is>
       </c>
       <c r="C321" s="2" t="inlineStr">
         <is>
-          <t>Người xem</t>
+          <t>Lưu</t>
         </is>
       </c>
     </row>
     <row r="322" ht="18" customHeight="1">
       <c r="A322" s="2" t="inlineStr">
         <is>
-          <t>room.settings.save</t>
+          <t>room-invite.messages.title</t>
         </is>
       </c>
       <c r="B322" s="2" t="inlineStr">
         <is>
-          <t>Save</t>
+          <t>Room Invitation</t>
         </is>
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>Lưu</t>
+          <t>Lời mời vào phòng</t>
         </is>
       </c>
     </row>
     <row r="323" ht="54" customHeight="1">
       <c r="A323" s="2" t="inlineStr">
         <is>
-          <t>room-invite.messages.title</t>
+          <t>start-game.messages.success</t>
         </is>
       </c>
       <c r="B323" s="2" t="inlineStr">
         <is>
-          <t>Room Invitation</t>
+          <t>Game started successfully</t>
         </is>
       </c>
       <c r="C323" s="2" t="inlineStr">
         <is>
-          <t>Lời mời vào phòng</t>
+          <t>Bắt đầu trò chơi thành công</t>
         </is>
       </c>
     </row>
     <row r="324" ht="18" customHeight="1">
       <c r="A324" s="2" t="inlineStr">
         <is>
-          <t>start-game.messages.success</t>
+          <t>start-game.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B324" s="2" t="inlineStr">
         <is>
-          <t>Game started successfully</t>
+          <t>Internal server error while starting game</t>
         </is>
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>Bắt đầu trò chơi thành công</t>
+          <t>Lỗi máy chủ nội bộ khi bắt đầu trò chơi</t>
         </is>
       </c>
     </row>
     <row r="325" ht="72" customHeight="1">
       <c r="A325" s="2" t="inlineStr">
         <is>
-          <t>start-game.messages.internal-server-error</t>
+          <t>start-game.messages.invalid-room-id</t>
         </is>
       </c>
       <c r="B325" s="2" t="inlineStr">
         <is>
-          <t>Internal server error while starting game</t>
+          <t>Field 'id' is required and must be a positive integer</t>
         </is>
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ khi bắt đầu trò chơi</t>
+          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
         </is>
       </c>
     </row>
     <row r="326" ht="18" customHeight="1">
       <c r="A326" s="2" t="inlineStr">
         <is>
-          <t>start-game.messages.invalid-room-id</t>
+          <t>start-game.messages.invalid-difficulty</t>
         </is>
       </c>
       <c r="B326" s="2" t="inlineStr">
         <is>
-          <t>Field 'id' is required and must be a positive integer</t>
+          <t>Bot difficulty must be between 1 and 5</t>
         </is>
       </c>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>Trường 'id' là bắt buộc và phải là số nguyên dương</t>
+          <t>Độ khó của bot phải từ 1 đến 5</t>
         </is>
       </c>
     </row>
     <row r="327" ht="90" customHeight="1">
       <c r="A327" s="2" t="inlineStr">
         <is>
-          <t>start-game.messages.invalid-difficulty</t>
+          <t>start-game.messages.room-not-found</t>
         </is>
       </c>
       <c r="B327" s="2" t="inlineStr">
         <is>
-          <t>Bot difficulty must be between 1 and 5</t>
+          <t>Room not found</t>
         </is>
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>Độ khó của bot phải từ 1 đến 5</t>
+          <t>Không tìm thấy phòng</t>
         </is>
       </c>
     </row>
     <row r="328" ht="18" customHeight="1">
       <c r="A328" s="2" t="inlineStr">
         <is>
-          <t>start-game.messages.room-not-found</t>
+          <t>start-game.messages.forbidden</t>
         </is>
       </c>
       <c r="B328" s="2" t="inlineStr">
         <is>
-          <t>Room not found</t>
+          <t>Only the room host can start the game</t>
         </is>
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy phòng</t>
+          <t>Chỉ chủ phòng mới có thể bắt đầu trò chơi</t>
         </is>
       </c>
     </row>
     <row r="329" ht="72" customHeight="1">
       <c r="A329" s="2" t="inlineStr">
         <is>
-          <t>start-game.messages.forbidden</t>
+          <t>start-game.messages.insufficient-amount</t>
         </is>
       </c>
       <c r="B329" s="2" t="inlineStr">
         <is>
-          <t>Only the room host can start the game</t>
+          <t>You do not have enough balance to start a game with this bet</t>
         </is>
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>Chỉ chủ phòng mới có thể bắt đầu trò chơi</t>
+          <t>Bạn không còn đủ amount để start room</t>
         </is>
       </c>
     </row>
     <row r="330" ht="54" customHeight="1">
       <c r="A330" s="2" t="inlineStr">
         <is>
-          <t>start-game.messages.insufficient-amount</t>
+          <t>start-game.messages.requester-must-pick-team</t>
         </is>
       </c>
       <c r="B330" s="2" t="inlineStr">
         <is>
-          <t>You do not have enough balance to start a game with this bet</t>
+          <t>You must select a team before starting a game with bot</t>
         </is>
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>Bạn không còn đủ amount để start room</t>
+          <t>Bạn phải chọn team trước khi bắt đầu trò chơi với bot</t>
         </is>
       </c>
     </row>
     <row r="331" ht="54" customHeight="1">
       <c r="A331" s="2" t="inlineStr">
         <is>
-          <t>start-game.messages.requester-must-pick-team</t>
+          <t>update-room.messages.success</t>
         </is>
       </c>
       <c r="B331" s="2" t="inlineStr">
         <is>
-          <t>You must select a team before starting a game with bot</t>
+          <t>Room updated successfully</t>
         </is>
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>Bạn phải chọn team trước khi bắt đầu trò chơi với bot</t>
+          <t>Cập nhật phòng thành công</t>
         </is>
       </c>
     </row>
     <row r="332" ht="54" customHeight="1">
       <c r="A332" s="2" t="inlineStr">
         <is>
-          <t>update-room.messages.success</t>
+          <t>update-room.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B332" s="2" t="inlineStr">
         <is>
-          <t>Room updated successfully</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>Cập nhật phòng thành công</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="333" ht="90" customHeight="1">
       <c r="A333" s="2" t="inlineStr">
         <is>
-          <t>update-room.messages.internal-server-error</t>
+          <t>update-room.messages.invalid-room-id</t>
         </is>
       </c>
       <c r="B333" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Invalid room ID</t>
         </is>
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>ID phòng không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="334" ht="54" customHeight="1">
       <c r="A334" s="2" t="inlineStr">
         <is>
-          <t>update-room.messages.invalid-room-id</t>
+          <t>update-room.messages.invalid-time-limit</t>
         </is>
       </c>
       <c r="B334" s="2" t="inlineStr">
         <is>
-          <t>Invalid room ID</t>
+          <t>Invalid time limit</t>
         </is>
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>ID phòng không hợp lệ</t>
+          <t>Thời gian không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="335" ht="36" customHeight="1">
       <c r="A335" s="2" t="inlineStr">
         <is>
-          <t>update-room.messages.invalid-time-limit</t>
+          <t>update-room.messages.invalid-time-increment</t>
         </is>
       </c>
       <c r="B335" s="2" t="inlineStr">
         <is>
-          <t>Invalid time limit</t>
+          <t>Invalid bonus per move</t>
         </is>
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>Thời gian không hợp lệ</t>
+          <t>Thời gian cộng mỗi nước không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="336" ht="18" customHeight="1">
       <c r="A336" s="2" t="inlineStr">
         <is>
-          <t>update-room.messages.invalid-time-increment</t>
+          <t>update-room.messages.invalid-time-per-move</t>
         </is>
       </c>
       <c r="B336" s="2" t="inlineStr">
         <is>
-          <t>Invalid bonus per move</t>
+          <t>Invalid time per move</t>
         </is>
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>Thời gian cộng mỗi nước không hợp lệ</t>
+          <t>Thời gian mỗi nước không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="337" ht="36" customHeight="1">
       <c r="A337" s="2" t="inlineStr">
         <is>
-          <t>update-room.messages.invalid-time-per-move</t>
+          <t>update-room.messages.name-required</t>
         </is>
       </c>
       <c r="B337" s="2" t="inlineStr">
         <is>
-          <t>Invalid time per move</t>
+          <t>Room name is required</t>
         </is>
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>Thời gian mỗi nước không hợp lệ</t>
+          <t>Tên phòng không được để trống</t>
         </is>
       </c>
     </row>
     <row r="338" ht="36" customHeight="1">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>update-room.messages.name-required</t>
+          <t>update-room.messages.room-not-found</t>
         </is>
       </c>
       <c r="B338" s="2" t="inlineStr">
         <is>
-          <t>Room name is required</t>
+          <t>Room not found</t>
         </is>
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
-          <t>Tên phòng không được để trống</t>
+          <t>Không tìm thấy phòng</t>
         </is>
       </c>
     </row>
     <row r="339" ht="72" customHeight="1">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t>update-room.messages.room-not-found</t>
+          <t>update-room.messages.forbidden</t>
         </is>
       </c>
       <c r="B339" s="2" t="inlineStr">
         <is>
-          <t>Room not found</t>
+          <t>You are not the host of this room</t>
         </is>
       </c>
       <c r="C339" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy phòng</t>
+          <t>Bạn không phải chủ phòng</t>
         </is>
       </c>
     </row>
     <row r="340" ht="54" customHeight="1">
       <c r="A340" s="2" t="inlineStr">
         <is>
-          <t>update-room.messages.forbidden</t>
+          <t>draw-game.messages.invalid-game-id</t>
         </is>
       </c>
       <c r="B340" s="2" t="inlineStr">
         <is>
-          <t>You are not the host of this room</t>
+          <t>Invalid game ID</t>
         </is>
       </c>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>Bạn không phải chủ phòng</t>
+          <t>ID trò chơi không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="341" ht="54" customHeight="1">
       <c r="A341" s="2" t="inlineStr">
         <is>
-          <t>draw-game.messages.invalid-game-id</t>
+          <t>draw-game.messages.game-not-found</t>
         </is>
       </c>
       <c r="B341" s="2" t="inlineStr">
         <is>
-          <t>Invalid game ID</t>
+          <t>Game not found</t>
         </is>
       </c>
       <c r="C341" s="2" t="inlineStr">
         <is>
-          <t>ID trò chơi không hợp lệ</t>
+          <t>Không tìm thấy trò chơi</t>
         </is>
       </c>
     </row>
     <row r="342" ht="90" customHeight="1">
       <c r="A342" s="2" t="inlineStr">
         <is>
-          <t>draw-game.messages.game-not-found</t>
+          <t>draw-game.messages.forbidden</t>
         </is>
       </c>
       <c r="B342" s="2" t="inlineStr">
         <is>
-          <t>Game not found</t>
+          <t>You are not in this room</t>
         </is>
       </c>
       <c r="C342" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy trò chơi</t>
+          <t>Bạn không có trong phòng này</t>
         </is>
       </c>
     </row>
     <row r="343" ht="54" customHeight="1">
       <c r="A343" s="2" t="inlineStr">
         <is>
-          <t>draw-game.messages.forbidden</t>
+          <t>draw-game.messages.game-history-not-found</t>
         </is>
       </c>
       <c r="B343" s="2" t="inlineStr">
         <is>
-          <t>You are not in this room</t>
+          <t>Game history not found</t>
         </is>
       </c>
       <c r="C343" s="2" t="inlineStr">
         <is>
-          <t>Bạn không có trong phòng này</t>
+          <t>Không tìm thấy lịch sử trò chơi</t>
         </is>
       </c>
     </row>
     <row r="344" ht="18" customHeight="1">
       <c r="A344" s="2" t="inlineStr">
         <is>
-          <t>draw-game.messages.game-history-not-found</t>
+          <t>draw-game.messages.game-already-finished</t>
         </is>
       </c>
       <c r="B344" s="2" t="inlineStr">
         <is>
-          <t>Game history not found</t>
+          <t>Game is already finished</t>
         </is>
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy lịch sử trò chơi</t>
+          <t>Trò chơi đã kết thúc</t>
         </is>
       </c>
     </row>
     <row r="345" ht="18" customHeight="1">
       <c r="A345" s="2" t="inlineStr">
         <is>
-          <t>draw-game.messages.game-already-finished</t>
+          <t>draw-game.messages.success</t>
         </is>
       </c>
       <c r="B345" s="2" t="inlineStr">
         <is>
-          <t>Game is already finished</t>
+          <t>Draw game successfully</t>
         </is>
       </c>
       <c r="C345" s="2" t="inlineStr">
         <is>
-          <t>Trò chơi đã kết thúc</t>
+          <t>Hòa cờ thành công</t>
         </is>
       </c>
     </row>
     <row r="346" ht="36" customHeight="1">
       <c r="A346" s="2" t="inlineStr">
         <is>
-          <t>draw-game.messages.success</t>
+          <t>draw-game.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B346" s="2" t="inlineStr">
         <is>
-          <t>Draw game successfully</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C346" s="2" t="inlineStr">
         <is>
-          <t>Hòa cờ thành công</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="347" ht="18" customHeight="1">
       <c r="A347" s="2" t="inlineStr">
         <is>
-          <t>draw-game.messages.internal-server-error</t>
+          <t>surrender.messages.game-already-finished</t>
         </is>
       </c>
       <c r="B347" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Game is already finished</t>
         </is>
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>Trò chơi đã kết thúc</t>
         </is>
       </c>
     </row>
     <row r="348" ht="18" customHeight="1">
       <c r="A348" s="2" t="inlineStr">
         <is>
-          <t>surrender.messages.game-already-finished</t>
+          <t>surrender.messages.game-history-not-found</t>
         </is>
       </c>
       <c r="B348" s="2" t="inlineStr">
         <is>
-          <t>Game is already finished</t>
+          <t>Game history not found</t>
         </is>
       </c>
       <c r="C348" s="2" t="inlineStr">
         <is>
-          <t>Trò chơi đã kết thúc</t>
+          <t>Không tìm thấy lịch sử trò chơi</t>
         </is>
       </c>
     </row>
     <row r="349" ht="36" customHeight="1">
       <c r="A349" s="2" t="inlineStr">
         <is>
-          <t>surrender.messages.game-history-not-found</t>
+          <t>surrender.messages.game-not-found</t>
         </is>
       </c>
       <c r="B349" s="2" t="inlineStr">
         <is>
-          <t>Game history not found</t>
+          <t>Game not found</t>
         </is>
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy lịch sử trò chơi</t>
+          <t>Không tìm thấy trò chơi</t>
         </is>
       </c>
     </row>
     <row r="350" ht="18" customHeight="1">
       <c r="A350" s="2" t="inlineStr">
         <is>
-          <t>surrender.messages.game-not-found</t>
+          <t>surrender.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B350" s="2" t="inlineStr">
         <is>
-          <t>Game not found</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy trò chơi</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="351" ht="36" customHeight="1">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t>surrender.messages.internal-server-error</t>
+          <t>surrender.messages.invalid-game-id</t>
         </is>
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Invalid game ID</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>ID trò chơi không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="352" ht="18" customHeight="1">
       <c r="A352" s="2" t="inlineStr">
         <is>
-          <t>surrender.messages.invalid-game-id</t>
+          <t>surrender.messages.invalid-surrender-player</t>
         </is>
       </c>
       <c r="B352" s="2" t="inlineStr">
         <is>
-          <t>Invalid game ID</t>
+          <t>You are not a player in this game</t>
         </is>
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>ID trò chơi không hợp lệ</t>
+          <t>Bạn không phải là người chơi trong trò chơi này</t>
         </is>
       </c>
     </row>
     <row r="353" ht="18" customHeight="1">
       <c r="A353" s="2" t="inlineStr">
         <is>
-          <t>surrender.messages.invalid-surrender-player</t>
+          <t>surrender.messages.opponent-not-found</t>
         </is>
       </c>
       <c r="B353" s="2" t="inlineStr">
         <is>
-          <t>You are not a player in this game</t>
+          <t>Opponent not found</t>
         </is>
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>Bạn không phải là người chơi trong trò chơi này</t>
+          <t>Không tìm thấy đối thủ</t>
         </is>
       </c>
     </row>
     <row r="354" ht="18" customHeight="1">
       <c r="A354" s="2" t="inlineStr">
         <is>
-          <t>surrender.messages.opponent-not-found</t>
+          <t>surrender.messages.success</t>
         </is>
       </c>
       <c r="B354" s="2" t="inlineStr">
         <is>
-          <t>Opponent not found</t>
+          <t>Surrendered</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy đối thủ</t>
+          <t>Đã đầu hàng</t>
         </is>
       </c>
     </row>
     <row r="355" ht="18" customHeight="1">
       <c r="A355" s="2" t="inlineStr">
         <is>
-          <t>surrender.messages.success</t>
+          <t>undo.messages.invalid-game-id</t>
         </is>
       </c>
       <c r="B355" s="2" t="inlineStr">
         <is>
-          <t>Surrendered</t>
+          <t>Invalid game ID</t>
         </is>
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>Đã đầu hàng</t>
+          <t>ID trò chơi không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="356" ht="18" customHeight="1">
       <c r="A356" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.invalid-game-id</t>
+          <t>undo.messages.unauthorized</t>
         </is>
       </c>
       <c r="B356" s="2" t="inlineStr">
         <is>
-          <t>Invalid game ID</t>
+          <t>Unauthorized</t>
         </is>
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>ID trò chơi không hợp lệ</t>
+          <t>Không được phép truy cập</t>
         </is>
       </c>
     </row>
     <row r="357" ht="17" customHeight="1">
       <c r="A357" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.unauthorized</t>
+          <t>undo.messages.game-not-found</t>
         </is>
       </c>
       <c r="B357" s="2" t="inlineStr">
         <is>
-          <t>Unauthorized</t>
+          <t>Game not found</t>
         </is>
       </c>
       <c r="C357" s="2" t="inlineStr">
         <is>
-          <t>Không được phép truy cập</t>
+          <t>Không tìm thấy trò chơi</t>
         </is>
       </c>
     </row>
     <row r="358" ht="18" customHeight="1">
       <c r="A358" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.game-not-found</t>
+          <t>undo.messages.not-in-game</t>
         </is>
       </c>
       <c r="B358" s="2" t="inlineStr">
         <is>
-          <t>Game not found</t>
+          <t>You are not part of this game</t>
         </is>
       </c>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>Không tìm thấy trò chơi</t>
+          <t>Bạn không phải là người chơi trong trò chơi này</t>
         </is>
       </c>
     </row>
     <row r="359" ht="18" customHeight="1">
       <c r="A359" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.not-in-game</t>
+          <t>undo.messages.not-in-room</t>
         </is>
       </c>
       <c r="B359" s="2" t="inlineStr">
         <is>
-          <t>You are not part of this game</t>
+          <t>You are not in this room</t>
         </is>
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
-          <t>Bạn không phải là người chơi trong trò chơi này</t>
+          <t>Bạn không trong phòng này</t>
         </is>
       </c>
     </row>
     <row r="360" ht="18" customHeight="1">
       <c r="A360" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.not-in-room</t>
+          <t>undo.messages.pve-only</t>
         </is>
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>You are not in this room</t>
+          <t>Undo is only available in PvE rooms</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>Bạn không trong phòng này</t>
+          <t>Hoàn tác chỉ khả dụng trong phòng PvE</t>
         </is>
       </c>
     </row>
     <row r="361" ht="18" customHeight="1">
       <c r="A361" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.pve-only</t>
+          <t>undo.messages.spectator-cannot-undo</t>
         </is>
       </c>
       <c r="B361" s="2" t="inlineStr">
         <is>
-          <t>Undo is only available in PvE rooms</t>
+          <t>Spectators cannot undo moves</t>
         </is>
       </c>
       <c r="C361" s="2" t="inlineStr">
         <is>
-          <t>Hoàn tác chỉ khả dụng trong phòng PvE</t>
+          <t>Người xem không thể hoàn tác nước đi</t>
         </is>
       </c>
     </row>
     <row r="362" ht="18" customHeight="1">
       <c r="A362" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.spectator-cannot-undo</t>
+          <t>undo.messages.no-moves</t>
         </is>
       </c>
       <c r="B362" s="2" t="inlineStr">
         <is>
-          <t>Spectators cannot undo moves</t>
+          <t>No moves to undo</t>
         </is>
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>Người xem không thể hoàn tác nước đi</t>
+          <t>Không có nước đi để hoàn tác</t>
         </is>
       </c>
     </row>
     <row r="363" ht="18" customHeight="1">
       <c r="A363" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.no-moves</t>
+          <t>undo.messages.delete-failed</t>
         </is>
       </c>
       <c r="B363" s="2" t="inlineStr">
         <is>
-          <t>No moves to undo</t>
+          <t>Failed to undo move</t>
         </is>
       </c>
       <c r="C363" s="2" t="inlineStr">
         <is>
-          <t>Không có nước đi để hoàn tác</t>
+          <t>Không thể hoàn tác nước đi</t>
         </is>
       </c>
     </row>
     <row r="364" ht="17" customHeight="1">
       <c r="A364" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.delete-failed</t>
+          <t>undo.messages.undo-limit-exceeded</t>
         </is>
       </c>
       <c r="B364" s="2" t="inlineStr">
         <is>
-          <t>Failed to undo move</t>
+          <t>Maximum 3 undo per game exceeded</t>
         </is>
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>Không thể hoàn tác nước đi</t>
+          <t>Đã đạt tối đa 3 lần hoàn tác trong trò chơi</t>
         </is>
       </c>
     </row>
     <row r="365" ht="17" customHeight="1">
       <c r="A365" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.undo-limit-exceeded</t>
+          <t>undo.messages.success</t>
         </is>
       </c>
       <c r="B365" s="2" t="inlineStr">
         <is>
-          <t>Maximum 3 undo per game exceeded</t>
+          <t>Move undone successfully</t>
         </is>
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>Đã đạt tối đa 3 lần hoàn tác trong trò chơi</t>
+          <t>Hoàn tác nước đi thành công</t>
         </is>
       </c>
     </row>
     <row r="366" ht="17" customHeight="1">
       <c r="A366" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.success</t>
+          <t>undo.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B366" s="2" t="inlineStr">
         <is>
-          <t>Move undone successfully</t>
+          <t>Internal server error</t>
         </is>
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>Hoàn tác nước đi thành công</t>
+          <t>Lỗi máy chủ nội bộ</t>
         </is>
       </c>
     </row>
     <row r="367" ht="17" customHeight="1">
       <c r="A367" s="2" t="inlineStr">
         <is>
-          <t>undo.messages.internal-server-error</t>
+          <t>player-history.messages.invalid-user-id</t>
         </is>
       </c>
       <c r="B367" s="2" t="inlineStr">
         <is>
-          <t>Internal server error</t>
+          <t>Invalid user ID</t>
         </is>
       </c>
       <c r="C367" s="2" t="inlineStr">
         <is>
-          <t>Lỗi máy chủ nội bộ</t>
+          <t>ID người dùng không hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="368" ht="17" customHeight="1">
       <c r="A368" s="2" t="inlineStr">
         <is>
-          <t>player-history.messages.invalid-user-id</t>
+          <t>player-history.messages.success</t>
         </is>
       </c>
       <c r="B368" s="2" t="inlineStr">
         <is>
-          <t>Invalid user ID</t>
+          <t>Fetch game history successfully</t>
         </is>
       </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>ID người dùng không hợp lệ</t>
+          <t>Lấy lịch sử trò chơi thành công</t>
         </is>
       </c>
     </row>
     <row r="369" ht="17" customHeight="1">
       <c r="A369" s="2" t="inlineStr">
         <is>
-          <t>player-history.messages.success</t>
+          <t>validate-token.messages.success</t>
         </is>
       </c>
       <c r="B369" s="2" t="inlineStr">
         <is>
-          <t>Fetch game history successfully</t>
+          <t>Token is valid</t>
         </is>
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
-          <t>Lấy lịch sử trò chơi thành công</t>
+          <t>Token hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="370" ht="17" customHeight="1">
       <c r="A370" s="2" t="inlineStr">
         <is>
-          <t>validate-token.messages.success</t>
+          <t>guide.section.objective</t>
         </is>
       </c>
       <c r="B370" s="2" t="inlineStr">
         <is>
-          <t>Token is valid</t>
+          <t>Objective of the game</t>
         </is>
       </c>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>Token hợp lệ</t>
+          <t>Mục tiêu của trò chơi</t>
         </is>
       </c>
     </row>
     <row r="371" ht="17" customHeight="1">
       <c r="A371" s="2" t="inlineStr">
         <is>
-          <t>guide.section.objective</t>
+          <t>guide.section.pieces</t>
         </is>
       </c>
       <c r="B371" s="2" t="inlineStr">
         <is>
-          <t>Objective of the game</t>
+          <t>Pieces</t>
         </is>
       </c>
       <c r="C371" s="2" t="inlineStr">
         <is>
-          <t>Mục tiêu của trò chơi</t>
+          <t>Quân cờ</t>
         </is>
       </c>
     </row>
     <row r="372" ht="17" customHeight="1">
       <c r="A372" s="2" t="inlineStr">
         <is>
-          <t>guide.section.pieces</t>
+          <t>guide.section.moving-pieces</t>
         </is>
       </c>
       <c r="B372" s="2" t="inlineStr">
         <is>
-          <t>Pieces</t>
+          <t>Moving pieces</t>
         </is>
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>Quân cờ</t>
+          <t>Đi quân</t>
         </is>
       </c>
     </row>
     <row r="373" ht="17" customHeight="1">
       <c r="A373" s="2" t="inlineStr">
         <is>
-          <t>guide.section.moving-pieces</t>
+          <t>guide.section.capturing</t>
         </is>
       </c>
       <c r="B373" s="2" t="inlineStr">
         <is>
-          <t>Moving pieces</t>
+          <t>Capturing</t>
         </is>
       </c>
       <c r="C373" s="2" t="inlineStr">
         <is>
-          <t>Đi quân</t>
+          <t>Bắt quân</t>
         </is>
       </c>
     </row>
     <row r="374" ht="17" customHeight="1">
       <c r="A374" s="2" t="inlineStr">
         <is>
-          <t>guide.section.capturing</t>
+          <t>guide.section.check</t>
         </is>
       </c>
       <c r="B374" s="2" t="inlineStr">
         <is>
-          <t>Capturing</t>
+          <t>Check</t>
         </is>
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>Bắt quân</t>
+          <t>Chiếu tướng</t>
         </is>
       </c>
     </row>
     <row r="375" ht="17" customHeight="1">
       <c r="A375" s="2" t="inlineStr">
         <is>
-          <t>guide.section.check</t>
+          <t>guide.section.result</t>
         </is>
       </c>
       <c r="B375" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Result</t>
         </is>
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>Chiếu tướng</t>
+          <t>Kết quả</t>
         </is>
       </c>
     </row>
     <row r="376" ht="17" customHeight="1">
       <c r="A376" s="2" t="inlineStr">
         <is>
-          <t>guide.section.result</t>
+          <t>guide.table.piece</t>
         </is>
       </c>
       <c r="B376" s="2" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>Piece</t>
         </is>
       </c>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t>Kết quả</t>
+          <t>Quân</t>
         </is>
       </c>
     </row>
     <row r="377" ht="17" customHeight="1">
       <c r="A377" s="2" t="inlineStr">
         <is>
-          <t>guide.table.piece</t>
+          <t>guide.table.symbol</t>
         </is>
       </c>
       <c r="B377" s="2" t="inlineStr">
         <is>
-          <t>Piece</t>
+          <t>Symbol</t>
         </is>
       </c>
       <c r="C377" s="2" t="inlineStr">
         <is>
-          <t>Quân</t>
+          <t>Ký hiệu</t>
         </is>
       </c>
     </row>
     <row r="378" ht="17" customHeight="1">
       <c r="A378" s="2" t="inlineStr">
         <is>
-          <t>guide.table.symbol</t>
+          <t>guide.table.quantity</t>
         </is>
       </c>
       <c r="B378" s="2" t="inlineStr">
         <is>
-          <t>Symbol</t>
+          <t>Quantity</t>
         </is>
       </c>
       <c r="C378" s="2" t="inlineStr">
         <is>
-          <t>Ký hiệu</t>
+          <t>Số lượng</t>
         </is>
       </c>
     </row>
     <row r="379" ht="17" customHeight="1">
       <c r="A379" s="2" t="inlineStr">
         <is>
-          <t>guide.table.quantity</t>
+          <t>guide.objective.paragraph1</t>
         </is>
       </c>
       <c r="B379" s="2" t="inlineStr">
         <is>
-          <t>Quantity</t>
+          <t>A match is played between two players: one controls the Red pieces, and the other controls the Black pieces. The objective of each player is to use their pieces on the board to &lt;b&gt;checkmate&lt;/b&gt; the opponent's General, and win the game.</t>
         </is>
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
-          <t>Số lượng</t>
+          <t>Ván cờ được tiến hành giữa 2 đấu thủ, một người cầm Quân Đỏ, một người cầm Quân Đen. Mục đích của mỗi đấu thủ là tìm mọi cách sử dụng các quân trên bàn cờ để &lt;b&gt;chiếu bí Tướng&lt;/b&gt; của đối phương, giành thắng lợi.</t>
         </is>
       </c>
     </row>
     <row r="380" ht="17" customHeight="1">
       <c r="A380" s="2" t="inlineStr">
         <is>
-          <t>guide.objective.paragraph1</t>
+          <t>guide.pieces.paragraph1</t>
         </is>
       </c>
       <c r="B380" s="2" t="inlineStr">
         <is>
-          <t>A match is played between two players: one controls the Red pieces, and the other controls the Black pieces. The objective of each player is to use their pieces on the board to &lt;b&gt;checkmate&lt;/b&gt; the opponent's General, and win the game.</t>
+          <t>At the start of each game, there must be 32 pieces in total, consisting of &lt;b&gt;7 piece types&lt;/b&gt; split evenly between both sides: 16 Red pieces and 16 Black pieces. The 7 piece types with their symbols and quantities are as follows:</t>
         </is>
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>Ván cờ được tiến hành giữa 2 đấu thủ, một người cầm Quân Đỏ, một người cầm Quân Đen. Mục đích của mỗi đấu thủ là tìm mọi cách sử dụng các quân trên bàn cờ để &lt;b&gt;chiếu bí Tướng&lt;/b&gt; của đối phương, giành thắng lợi.</t>
+          <t>Mỗi ván cờ lúc bắt đầu phải có đủ 32 quân, gồm 7 loại chia đều cho mỗi bên gồm 16 quân Đỏ và 16 quân Đen. &lt;b&gt;7 loại quân&lt;/b&gt; có ký hiệu và số lượng như sau:</t>
         </is>
       </c>
     </row>
     <row r="381" ht="17" customHeight="1">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>guide.pieces.paragraph1</t>
+          <t>guide.piece.general</t>
         </is>
       </c>
       <c r="B381" s="2" t="inlineStr">
         <is>
-          <t>At the start of each game, there must be 32 pieces in total, consisting of &lt;b&gt;7 piece types&lt;/b&gt; split evenly between both sides: 16 Red pieces and 16 Black pieces. The 7 piece types with their symbols and quantities are as follows:</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C381" s="2" t="inlineStr">
         <is>
-          <t>Mỗi ván cờ lúc bắt đầu phải có đủ 32 quân, gồm 7 loại chia đều cho mỗi bên gồm 16 quân Đỏ và 16 quân Đen. &lt;b&gt;7 loại quân&lt;/b&gt; có ký hiệu và số lượng như sau:</t>
+          <t>Tướng</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>guide.piece.general</t>
+          <t>guide.piece.advisor</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Advisor</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>Tướng</t>
+          <t>Sĩ</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>guide.piece.advisor</t>
+          <t>guide.piece.elephant</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>Advisor</t>
+          <t>Elephant</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>Sĩ</t>
+          <t>Tượng</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>guide.piece.elephant</t>
+          <t>guide.piece.chariot</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>Elephant</t>
+          <t>Chariot</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>Tượng</t>
+          <t>Xe</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>guide.piece.chariot</t>
+          <t>guide.piece.horse</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>Chariot</t>
+          <t>Horse</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>Xe</t>
+          <t>Mã</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>guide.piece.horse</t>
+          <t>guide.piece.cannon</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>Horse</t>
+          <t>Cannon</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>Mã</t>
+          <t>Pháo</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>guide.piece.cannon</t>
+          <t>guide.piece.soldier</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Cannon</t>
+          <t>Soldier</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>Pháo</t>
+          <t>Tốt</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>guide.piece.soldier</t>
+          <t>guide.moving-pieces.paragraph1</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>Soldier</t>
+          <t>On each turn, each side may move only one of its own pieces according to the rules. The movement rules are as follows:</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Tốt</t>
+          <t>Mỗi nước đi, mỗi bên chỉ được di chuyển quân của mình theo đúng quy định. Quy định di chuyển của các quân như sau:</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>guide.moving-pieces.paragraph1</t>
+          <t>guide.general.paragraph1</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>On each turn, each side may move only one of its own pieces according to the rules. The movement rules are as follows:</t>
+          <t>General</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>Mỗi nước đi, mỗi bên chỉ được di chuyển quân của mình theo đúng quy định. Quy định di chuyển của các quân như sau:</t>
+          <t>Tướng</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>guide.general.paragraph1</t>
+          <t>guide.general.paragraph2</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Moves one step &lt;b&gt;horizontally or vertically&lt;/b&gt; within the palace. The two Generals may not face each other directly on the same file. If they are facing each other, there must be at least one piece of either side placed between them.</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>Tướng</t>
+          <t>Mỗi nước được đi một bước &lt;b&gt;ngang hoặc dọc&lt;/b&gt; tùy ý trong cung Tướng. Hai tướng của 2 bên không được đối mặt nhau trực tiếp trên cùng một đường thẳng. Nếu đối mặt, bắt buộc phải có quân của bất kỳ bên nào đứng che mặt.</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>guide.general.paragraph2</t>
+          <t>guide.advisor.paragraph1</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>Moves one step &lt;b&gt;horizontally or vertically&lt;/b&gt; within the palace. The two Generals may not face each other directly on the same file. If they are facing each other, there must be at least one piece of either side placed between them.</t>
+          <t>Advisor</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Mỗi nước được đi một bước &lt;b&gt;ngang hoặc dọc&lt;/b&gt; tùy ý trong cung Tướng. Hai tướng của 2 bên không được đối mặt nhau trực tiếp trên cùng một đường thẳng. Nếu đối mặt, bắt buộc phải có quân của bất kỳ bên nào đứng che mặt.</t>
+          <t>Sĩ</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>guide.advisor.paragraph1</t>
+          <t>guide.advisor.paragraph2</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>Advisor</t>
+          <t>Moves one step &lt;b&gt;diagonally&lt;/b&gt; within the palace.</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>Sĩ</t>
+          <t>Mỗi nước &lt;b&gt;đi chéo một bước&lt;/b&gt; trong cung Tướng.</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>guide.advisor.paragraph2</t>
+          <t>guide.elephant.paragraph1</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>Moves one step &lt;b&gt;diagonally&lt;/b&gt; within the palace.</t>
+          <t>Elephant</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Mỗi nước &lt;b&gt;đi chéo một bước&lt;/b&gt; trong cung Tướng.</t>
+          <t>Tượng</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>guide.elephant.paragraph1</t>
+          <t>guide.elephant.paragraph2</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>Elephant</t>
+          <t>Moves &lt;b&gt;two steps diagonally&lt;/b&gt; on its own side of the board and may not cross the river. If there is another piece on the midpoint of that diagonal path, the Elephant is blocked and cannot move.</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>Tượng</t>
+          <t>Mỗi nước &lt;b&gt;đi chéo hai bước&lt;/b&gt; tại trận địa bên mình, không được qua sông. Nếu ở giữa đường chéo đó có quân khác đứng thì quân Tượng bị cản, không đi được.</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>guide.elephant.paragraph2</t>
+          <t>guide.chariot.paragraph1</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;two steps diagonally&lt;/b&gt; on its own side of the board and may not cross the river. If there is another piece on the midpoint of that diagonal path, the Elephant is blocked and cannot move.</t>
+          <t>Chariot</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>Mỗi nước &lt;b&gt;đi chéo hai bước&lt;/b&gt; tại trận địa bên mình, không được qua sông. Nếu ở giữa đường chéo đó có quân khác đứng thì quân Tượng bị cản, không đi được.</t>
+          <t>Xe</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>guide.chariot.paragraph1</t>
+          <t>guide.chariot.paragraph2</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>Chariot</t>
+          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; with no limit on distance, as long as no piece blocks the path.</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>Xe</t>
+          <t>Mỗi nước được &lt;b&gt;đi dọc hoặc đi ngang&lt;/b&gt;, không hạn chế số bước đi nếu không có quân khác cản đường.</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>guide.chariot.paragraph2</t>
+          <t>guide.horse.paragraph1</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; with no limit on distance, as long as no piece blocks the path.</t>
+          <t>Horse</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>Mỗi nước được &lt;b&gt;đi dọc hoặc đi ngang&lt;/b&gt;, không hạn chế số bước đi nếu không có quân khác cản đường.</t>
+          <t>Mã</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>guide.horse.paragraph1</t>
+          <t>guide.horse.paragraph2</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>Horse</t>
+          <t>Moves in an &lt;b&gt;L-shape&lt;/b&gt; (one step orthogonally then one step diagonally outward). If the adjacent orthogonal point is occupied by any piece, the Horse is blocked and cannot move.</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>Mã</t>
+          <t>Đi theo &lt;b&gt;đường chéo hình chữ nhật&lt;/b&gt; của hai ô vuông liền nhau. Nếu giao điểm liền kề bước thẳng dọc ngang có một quân khác đứng thì Mã bị cản, không đi được.</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>guide.horse.paragraph2</t>
+          <t>guide.cannon.paragraph1</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>Moves in an &lt;b&gt;L-shape&lt;/b&gt; (one step orthogonally then one step diagonally outward). If the adjacent orthogonal point is occupied by any piece, the Horse is blocked and cannot move.</t>
+          <t>Cannon</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>Đi theo &lt;b&gt;đường chéo hình chữ nhật&lt;/b&gt; của hai ô vuông liền nhau. Nếu giao điểm liền kề bước thẳng dọc ngang có một quân khác đứng thì Mã bị cản, không đi được.</t>
+          <t>Pháo</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>guide.cannon.paragraph1</t>
+          <t>guide.cannon.paragraph2</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>Cannon</t>
+          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; like a Chariot when not capturing. To capture, it must &lt;b&gt;jump over exactly one piece&lt;/b&gt; to reach its target. If there are zero or more than one pieces between the Cannon and the target, it cannot capture.</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>Pháo</t>
+          <t>Đi ngang hoặc dọc giống Xe khi không bắt quân. Để bắt quân, nó phải &lt;b&gt;nhảy qua đúng một quân khác&lt;/b&gt; để đến mục tiêu. Nếu không có hoặc có nhiều hơn một quân giữa Pháo và mục tiêu, nó không thể bắt quân.</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>guide.cannon.paragraph2</t>
+          <t>guide.soldier.paragraph1</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; like a Chariot when not capturing. To capture, it must &lt;b&gt;jump over exactly one piece&lt;/b&gt; to reach its target. If there are zero or more than one pieces between the Cannon and the target, it cannot capture.</t>
+          <t>Soldier</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>Đi ngang hoặc dọc giống Xe khi không bắt quân. Để bắt quân, nó phải &lt;b&gt;nhảy qua đúng một quân khác&lt;/b&gt; để đến mục tiêu. Nếu không có hoặc có nhiều hơn một quân giữa Pháo và mục tiêu, nó không thể bắt quân.</t>
+          <t>Tốt</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>guide.soldier.paragraph1</t>
+          <t>guide.soldier.paragraph2</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>Soldier</t>
+          <t>Moves &lt;b&gt;one step&lt;/b&gt; each turn. Before crossing the river, it can only move forward. After crossing the river, it may move &lt;b&gt;forward or sideways&lt;/b&gt;, but never backward.</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>Tốt</t>
+          <t>Mỗi nước đi &lt;b&gt;một bước&lt;/b&gt;. Khi chưa qua sông, Tốt chỉ được tiến. Khi Tốt đã qua sông được quyền &lt;b&gt;đi tiến và đi ngang&lt;/b&gt;, không được phép lùi.</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>guide.soldier.paragraph2</t>
+          <t>guide.capturing.paragraph1</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;one step&lt;/b&gt; each turn. Before crossing the river, it can only move forward. After crossing the river, it may move &lt;b&gt;forward or sideways&lt;/b&gt;, but never backward.</t>
+          <t>When a piece moves to an intersection occupied by an opponent's piece, it may &lt;b&gt;capture that piece&lt;/b&gt; and occupy its position.</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>Mỗi nước đi &lt;b&gt;một bước&lt;/b&gt;. Khi chưa qua sông, Tốt chỉ được tiến. Khi Tốt đã qua sông được quyền &lt;b&gt;đi tiến và đi ngang&lt;/b&gt;, không được phép lùi.</t>
+          <t>Khi một quân đi tới một giao điểm khác đã có quân đối phương đứng thì được quyền &lt;b&gt;bắt quân đó&lt;/b&gt;, đồng thời chiếm giữ vị trí quân bị bắt.</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>guide.capturing.paragraph1</t>
+          <t>guide.capturing.paragraph2</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>When a piece moves to an intersection occupied by an opponent's piece, it may &lt;b&gt;capture that piece&lt;/b&gt; and occupy its position.</t>
+          <t>You may not capture your own pieces. You may sacrifice your own pieces to be captured by the opponent, &lt;b&gt;except for the General&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>Khi một quân đi tới một giao điểm khác đã có quân đối phương đứng thì được quyền &lt;b&gt;bắt quân đó&lt;/b&gt;, đồng thời chiếm giữ vị trí quân bị bắt.</t>
+          <t>Không được bắt quân bên mình. Được phép cho đối phương bắt đầu quân mình chủ động hiến mình cho đối phương, &lt;b&gt;trừ Tướng&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>guide.capturing.paragraph2</t>
+          <t>guide.capturing.paragraph3</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>You may not capture your own pieces. You may sacrifice your own pieces to be captured by the opponent, &lt;b&gt;except for the General&lt;/b&gt;.</t>
+          <t>A captured piece is removed from the board. &lt;b&gt;Chasing one piece for more than 6 consecutive moves is not allowed&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>Không được bắt quân bên mình. Được phép cho đối phương bắt đầu quân mình chủ động hiến mình cho đối phương, &lt;b&gt;trừ Tướng&lt;/b&gt;.</t>
+          <t>Quân bị bắt phải bị loại và bị nhấc ra khỏi bàn cờ. &lt;b&gt;Không được đuổi 1 quân quá 6 nước cờ liên tiếp&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>guide.capturing.paragraph3</t>
+          <t>guide.check.paragraph1</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>A captured piece is removed from the board. &lt;b&gt;Chasing one piece for more than 6 consecutive moves is not allowed&lt;/b&gt;.</t>
+          <t>If a player makes a move that threatens to capture the opponent's General on the next move (by the same piece or another piece), it is called a &lt;b&gt;Check&lt;/b&gt;. The checked side must respond to avoid check. Otherwise, that side loses</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>Quân bị bắt phải bị loại và bị nhấc ra khỏi bàn cờ. &lt;b&gt;Không được đuổi 1 quân quá 6 nước cờ liên tiếp&lt;/b&gt;.</t>
+          <t>Nếu người chơi thực hiện một nước đi đe dọa bắt Tướng của đối phương ở nước đi tiếp theo (bằng chính quân cờ đó hoặc một quân cờ khác), thì đó được gọi là &lt;b&gt;Chiếu&lt;/b&gt;. Bên bị chiếu phải đáp trả để tránh bị chiếu. Nếu không sẽ bị xử thua</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>guide.check.paragraph1</t>
+          <t>guide.check.paragraph2</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>If a player makes a move that threatens to capture the opponent's General on the next move (by the same piece or another piece), it is called a &lt;b&gt;Check&lt;/b&gt;. The checked side must respond to avoid check. Otherwise, that side loses</t>
+          <t>When the General is checked from any direction (including from behind), the checked side may respond in one of the following ways:</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>Nếu người chơi thực hiện một nước đi đe dọa bắt Tướng của đối phương ở nước đi tiếp theo (bằng chính quân cờ đó hoặc một quân cờ khác), thì đó được gọi là &lt;b&gt;Chiếu&lt;/b&gt;. Bên bị chiếu phải đáp trả để tránh bị chiếu. Nếu không sẽ bị xử thua</t>
+          <t>Tướng bị chiếu từ cả bốn hướng (bị chiếu cả từ phía sau) có thể ứng phó với nước chiếu tướng bằng một trong các cách sau:</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>guide.check.paragraph2</t>
+          <t>guide.check.paragraph3</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>When the General is checked from any direction (including from behind), the checked side may respond in one of the following ways:</t>
+          <t>Move the General to another position to escape check</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Tướng bị chiếu từ cả bốn hướng (bị chiếu cả từ phía sau) có thể ứng phó với nước chiếu tướng bằng một trong các cách sau:</t>
+          <t>Di chuyển tướng sang vị trí khác để tránh nước chiếu</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>guide.check.paragraph3</t>
+          <t>guide.check.paragraph4</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>Move the General to another position to escape check</t>
+          <t>Capture the checking piece</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>Di chuyển tướng sang vị trí khác để tránh nước chiếu</t>
+          <t>Bắt quân đang chiếu</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>guide.check.paragraph4</t>
+          <t>guide.check.paragraph5</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>Capture the checking piece</t>
+          <t>Block the checking line with another piece to protect the General</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>Bắt quân đang chiếu</t>
+          <t>Dùng quân khác cản quân chiếu, đi quân che đỡ cho tướng</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>guide.check.paragraph5</t>
+          <t>guide.check.paragraph6</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>Block the checking line with another piece to protect the General</t>
+          <t>Repeatedly checking for more than 6 consecutive moves is not allowed</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>Dùng quân khác cản quân chiếu, đi quân che đỡ cho tướng</t>
+          <t>Không được chiếu tướng quá 6 nước cờ liên tiếp</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>guide.check.paragraph6</t>
+          <t>guide.result.paragraph1</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>Repeatedly checking for more than 6 consecutive moves is not allowed</t>
+          <t>When one side gives Check and the other side has no legal way to protect the General, it is called a &lt;b&gt;Checkmate&lt;/b&gt;. The side that delivers Checkmate wins.</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>Không được chiếu tướng quá 6 nước cờ liên tiếp</t>
+          <t>Khi một bên chiếu Tướng mà bên còn lại không thể làm gì để bảo vệ Tướng thì được gọi là &lt;b&gt;Chiếu Hết&lt;/b&gt;, bên thực hiện được Chiếu Hết sẽ giành chiến thắng.</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>guide.result.paragraph1</t>
+          <t>guide.result.paragraph2</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>When one side gives Check and the other side has no legal way to protect the General, it is called a &lt;b&gt;Checkmate&lt;/b&gt;. The side that delivers Checkmate wins.</t>
+          <t>If a player runs out of time for a single move (for example: 90s) without moving, the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>Khi một bên chiếu Tướng mà bên còn lại không thể làm gì để bảo vệ Tướng thì được gọi là &lt;b&gt;Chiếu Hết&lt;/b&gt;, bên thực hiện được Chiếu Hết sẽ giành chiến thắng.</t>
+          <t>Khi hết thời gian một nước đi (ví dụ: 90s) mà vẫn chưa di chuyển quân thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>guide.result.paragraph2</t>
+          <t>guide.result.paragraph3</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>If a player runs out of time for a single move (for example: 90s) without moving, the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
+          <t>If a player runs out of total game time (for example: 5 minutes or 10 minutes), the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>Khi hết thời gian một nước đi (ví dụ: 90s) mà vẫn chưa di chuyển quân thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
+          <t>Khi một bên hết thời gian ván đấu (ví dụ: 5 phút, 10 phút) thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>guide.result.paragraph3</t>
+          <t>guide.result.paragraph4</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>If a player runs out of total game time (for example: 5 minutes or 10 minutes), the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
+          <t>If both sides have no pieces that have crossed the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;. If one side still has pieces across the river but runs out of time, while the other side still has time but has no pieces across the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>Khi một bên hết thời gian ván đấu (ví dụ: 5 phút, 10 phút) thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
+          <t>Khi cả 2 bên đều không còn quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;. Khi một bên còn quân qua sông nhưng cạn thời gian, một bên còn thời gian nhưng hết quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>guide.result.paragraph4</t>
+          <t>guide.result.paragraph5</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>If both sides have no pieces that have crossed the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;. If one side still has pieces across the river but runs out of time, while the other side still has time but has no pieces across the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
+          <t>Within 50 moves, if there is no capture and no Soldier advances by one square, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>Khi cả 2 bên đều không còn quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;. Khi một bên còn quân qua sông nhưng cạn thời gian, một bên còn thời gian nhưng hết quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
+          <t>Trong vòng 50 nước nếu không phát sinh nước bắt quân, Tốt không tiến 1 ô thì ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>guide.result.paragraph5</t>
+          <t>extra-money.title</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>Within 50 moves, if there is no capture and no Soldier advances by one square, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
+          <t>Daily tasks</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>Trong vòng 50 nước nếu không phát sinh nước bắt quân, Tốt không tiến 1 ô thì ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
+          <t>Kiếm tiền</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>extra-money.title</t>
+          <t>extra-money.tab.lucky-wheel</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>Daily tasks</t>
+          <t>Lucky Wheel</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>Kiếm tiền</t>
+          <t>Vòng Quay May Mắn</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>extra-money.tab.lucky-wheel</t>
+          <t>extra-money.tab.bonus-coin</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>Lucky Wheel</t>
+          <t>Bonus Coin</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>Vòng Quay May Mắn</t>
+          <t>Xu Thưởng</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>extra-money.tab.bonus-coin</t>
+          <t>extra-money.tab.daily-bonus</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>Bonus Coin</t>
+          <t>Daily Bonus</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>Xu Thưởng</t>
+          <t>Thưởng hàng ngày</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>extra-money.tab.daily-bonus</t>
+          <t>extra-money.bonus-coin.subtitle</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>Daily Bonus</t>
+          <t>Watch a short video to earn free coin</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>Thưởng hàng ngày</t>
+          <t>Xem video ngắn để nhận xu miễn phí</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.subtitle</t>
+          <t>extra-money.bonus-coin.next-in</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>Watch a short video to earn free coin</t>
+          <t>Next in:</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>Xem video ngắn để nhận xu miễn phí</t>
+          <t>Lượt kế tiếp:</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.next-in</t>
+          <t>extra-money.bonus-coin.collect</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>Next in:</t>
+          <t>Collect</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>Lượt kế tiếp:</t>
+          <t>Thu thập</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.collect</t>
+          <t>extra-money.bonus-coin.watch-video</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>Collect</t>
+          <t>Watch video</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>Thu thập</t>
+          <t>Xem video</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.watch-video</t>
+          <t>extra-money.daily-bonus.subtitle</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>Watch video</t>
+          <t>Login 7 days in a row to earn 4000 coin</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>Xem video</t>
+          <t>Đăng nhập 7 ngày liên tiếp để nhận 4000 xu</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>extra-money.daily-bonus.subtitle</t>
+          <t>extra-money.daily-bonus.day</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>Login 7 days in a row to earn 4000 coin</t>
+          <t>Day</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>Đăng nhập 7 ngày liên tiếp để nhận 4000 xu</t>
+          <t>Ngày</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>extra-money.daily-bonus.day</t>
+          <t>extra-money.reward-ad.loading</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>Day</t>
+          <t>Loading ad...</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>Ngày</t>
+          <t>Đang tải quảng cáo...</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.loading</t>
+          <t>extra-money.reward-ad.error</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>Loading ad...</t>
+          <t>Could not load the ad. Please try again.</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>Đang tải quảng cáo...</t>
+          <t>Không tải được quảng cáo. Vui lòng thử lại.</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.error</t>
+          <t>extra-money.reward-ad.retry</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>Could not load the ad. Please try again.</t>
+          <t>Try again</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>Không tải được quảng cáo. Vui lòng thử lại.</t>
+          <t>Thử lại</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.retry</t>
+          <t>extra-money.reward-ad.close</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>Try again</t>
+          <t>Close</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>Thử lại</t>
+          <t>Đóng</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.close</t>
+          <t>profile.button.save</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Save</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>Đóng</t>
+          <t>Lưu</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>profile.button.save</t>
+          <t>profile.button.cancel</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>Save</t>
+          <t>Cancel</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>Lưu</t>
+          <t>Huỷ</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>profile.button.cancel</t>
+          <t>change-password.title</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>Cancel</t>
+          <t>Change password</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>Huỷ</t>
+          <t>Đổi mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>change-password.title</t>
+          <t>change-password.current.label</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>Change password</t>
+          <t>Current password</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>Đổi mật khẩu</t>
+          <t>Mật khẩu hiện tại</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>change-password.current.label</t>
+          <t>change-password.current.placeholder</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>Current password</t>
+          <t>Enter current password</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>Mật khẩu hiện tại</t>
+          <t>Nhập mật khẩu hiện tại</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>change-password.current.placeholder</t>
+          <t>change-password.new.label</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>Enter current password</t>
+          <t>New password</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>Nhập mật khẩu hiện tại</t>
+          <t>Mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>change-password.new.label</t>
+          <t>change-password.new.placeholder</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>New password</t>
+          <t>Enter new password</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>Mật khẩu mới</t>
+          <t>Nhập mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>change-password.new.placeholder</t>
+          <t>change-password.confirm.label</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>Enter new password</t>
+          <t>Confirm new password</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>Nhập mật khẩu mới</t>
+          <t>Xác nhận mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>change-password.confirm.label</t>
+          <t>change-password.confirm.placeholder</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>Confirm new password</t>
+          <t>Re-enter new password</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>Xác nhận mật khẩu mới</t>
+          <t>Nhập lại mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>change-password.confirm.placeholder</t>
+          <t>change-password.confirm.mismatch</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>Re-enter new password</t>
+          <t>Passwords do not match</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>Nhập lại mật khẩu mới</t>
+          <t>Mật khẩu xác nhận không khớp</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>change-password.confirm.mismatch</t>
+          <t>change-password.show</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>Passwords do not match</t>
+          <t>Show password</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>Mật khẩu xác nhận không khớp</t>
+          <t>Hiện mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>change-password.show</t>
+          <t>change-password.hide</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>Show password</t>
+          <t>Hide password</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>Hiện mật khẩu</t>
+          <t>Ẩn mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>change-password.hide</t>
+          <t>change-password.submit</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>Hide password</t>
+          <t>Change password</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>Ẩn mật khẩu</t>
+          <t>Đổi mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>change-password.submit</t>
+          <t>change-password.submitting</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>Change password</t>
+          <t>Changing...</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>Đổi mật khẩu</t>
+          <t>Đang đổi...</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>change-password.submitting</t>
+          <t>change-password.messages.success</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>Changing...</t>
+          <t>Password changed successfully</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>Đang đổi...</t>
+          <t>Đổi mật khẩu thành công</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>change-password.messages.success</t>
+          <t>change-password.messages.missing-fields</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>Password changed successfully</t>
+          <t>Please fill in all fields</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>Đổi mật khẩu thành công</t>
+          <t>Vui lòng nhập đầy đủ thông tin</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>change-password.messages.missing-fields</t>
+          <t>change-password.messages.weak-password</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>Please fill in all fields</t>
+          <t>New password does not meet the requirements</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>Vui lòng nhập đầy đủ thông tin</t>
+          <t>Mật khẩu mới không đạt yêu cầu</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>change-password.messages.weak-password</t>
+          <t>change-password.messages.same-as-current</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>New password does not meet the requirements</t>
+          <t>New password must be different from the current one</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>Mật khẩu mới không đạt yêu cầu</t>
+          <t>Mật khẩu mới phải khác mật khẩu hiện tại</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>change-password.messages.same-as-current</t>
+          <t>change-password.messages.incorrect-current-password</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>New password must be different from the current one</t>
+          <t>Current password is incorrect</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>Mật khẩu mới phải khác mật khẩu hiện tại</t>
+          <t>Mật khẩu hiện tại không đúng</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>change-password.messages.incorrect-current-password</t>
+          <t>change-password.messages.user-not-found</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>Current password is incorrect</t>
+          <t>User not found</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>Mật khẩu hiện tại không đúng</t>
+          <t>Không tìm thấy người dùng</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>change-password.messages.user-not-found</t>
+          <t>change-password.messages.unauthorized</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>User not found</t>
+          <t>Session expired. Please sign in again.</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>Không tìm thấy người dùng</t>
+          <t>Phiên đăng nhập đã hết hạn. Vui lòng đăng nhập lại.</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>change-password.messages.unauthorized</t>
+          <t>change-password.messages.internal-server-error</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>Session expired. Please sign in again.</t>
+          <t>Something went wrong. Please try again.</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>Phiên đăng nhập đã hết hạn. Vui lòng đăng nhập lại.</t>
+          <t>Đã có lỗi xảy ra. Vui lòng thử lại.</t>
         </is>
       </c>
     </row>
     <row r="453">
-      <c r="A453" t="inlineStr">
-        <is>
-          <t>change-password.messages.internal-server-error</t>
-        </is>
-      </c>
-      <c r="B453" t="inlineStr">
-        <is>
-          <t>Something went wrong. Please try again.</t>
-        </is>
-      </c>
-      <c r="C453" t="inlineStr">
-        <is>
-          <t>Đã có lỗi xảy ra. Vui lòng thử lại.</t>
-        </is>
-      </c>
+      <c r="A453" t="inlineStr"/>
+      <c r="B453" t="inlineStr"/>
+      <c r="C453" t="inlineStr"/>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr"/>
@@ -8123,11 +8111,6 @@
       <c r="A471" t="inlineStr"/>
       <c r="B471" t="inlineStr"/>
       <c r="C471" t="inlineStr"/>
-    </row>
-    <row r="472">
-      <c r="A472" t="inlineStr"/>
-      <c r="B472" t="inlineStr"/>
-      <c r="C472" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
- update rules and re-define language keys - fix deploy script
</commit_message>
<xml_diff>
--- a/tools/languages.xlsx
+++ b/tools/languages.xlsx
@@ -325,7 +325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C471"/>
+  <dimension ref="A1:C472"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1247,7 +1247,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Cầm hoà đối thủ khi chỉ còn tướng</t>
+          <t>Cầm hoà đối thủ khi chỉ còn vua</t>
         </is>
       </c>
     </row>
@@ -1764,17 +1764,17 @@
     <row r="85" ht="18" customHeight="1">
       <c r="A85" s="1" t="inlineStr">
         <is>
-          <t>dashboard.popup.red-first</t>
+          <t>dashboard.popup.white-first</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Red first</t>
+          <t>White first</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Đỏ tiên</t>
+          <t>Trắng tiên</t>
         </is>
       </c>
     </row>
@@ -2291,34 +2291,34 @@
     <row r="116" ht="18" customHeight="1">
       <c r="A116" s="1" t="inlineStr">
         <is>
-          <t>game.general.captured</t>
+          <t>game.king.checkmated</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>General has been captured. Room over</t>
+          <t>King is checkmated. Game over</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>Tướng đã bị bắt. Game kết thúc</t>
+          <t>Vua đã bị chiếu bí. Ván cờ kết thúc</t>
         </is>
       </c>
     </row>
     <row r="117" ht="18" customHeight="1">
       <c r="A117" s="1" t="inlineStr">
         <is>
-          <t>game.general.in-check</t>
+          <t>game.king.in-check</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>Your general is under attack</t>
+          <t>Your king is in check</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>Tướng của bạn đang bị chiếu</t>
+          <t>Vua của bạn đang bị chiếu</t>
         </is>
       </c>
     </row>
@@ -6687,7 +6687,7 @@
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>Chiếu tướng</t>
+          <t>Chiếu</t>
         </is>
       </c>
     </row>
@@ -6767,12 +6767,12 @@
       </c>
       <c r="B379" s="2" t="inlineStr">
         <is>
-          <t>A match is played between two players: one controls the Red pieces, and the other controls the Black pieces. The objective of each player is to use their pieces on the board to &lt;b&gt;checkmate&lt;/b&gt; the opponent's General, and win the game.</t>
+          <t>A chess game is played between two players: White and Black. The goal is to &lt;b&gt;checkmate&lt;/b&gt; the opponent's King.</t>
         </is>
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
-          <t>Ván cờ được tiến hành giữa 2 đấu thủ, một người cầm Quân Đỏ, một người cầm Quân Đen. Mục đích của mỗi đấu thủ là tìm mọi cách sử dụng các quân trên bàn cờ để &lt;b&gt;chiếu bí Tướng&lt;/b&gt; của đối phương, giành thắng lợi.</t>
+          <t>Một ván cờ vua được chơi giữa hai bên: Trắng và Đen. Mục tiêu là &lt;b&gt;chiếu bí&lt;/b&gt; Vua của đối phương.</t>
         </is>
       </c>
     </row>
@@ -6784,58 +6784,58 @@
       </c>
       <c r="B380" s="2" t="inlineStr">
         <is>
-          <t>At the start of each game, there must be 32 pieces in total, consisting of &lt;b&gt;7 piece types&lt;/b&gt; split evenly between both sides: 16 Red pieces and 16 Black pieces. The 7 piece types with their symbols and quantities are as follows:</t>
+          <t>A standard game starts with 32 pieces in total (16 per side), with &lt;b&gt;6 piece types&lt;/b&gt;: King, Queen, Rook, Bishop, Knight, and Pawn.</t>
         </is>
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>Mỗi ván cờ lúc bắt đầu phải có đủ 32 quân, gồm 7 loại chia đều cho mỗi bên gồm 16 quân Đỏ và 16 quân Đen. &lt;b&gt;7 loại quân&lt;/b&gt; có ký hiệu và số lượng như sau:</t>
+          <t>Một ván cờ tiêu chuẩn bắt đầu với 32 quân (mỗi bên 16 quân), gồm &lt;b&gt;6 loại quân&lt;/b&gt;: Vua, Hậu, Xe, Tượng, Mã và Tốt.</t>
         </is>
       </c>
     </row>
     <row r="381" ht="17" customHeight="1">
       <c r="A381" s="2" t="inlineStr">
         <is>
-          <t>guide.piece.general</t>
+          <t>guide.piece.king</t>
         </is>
       </c>
       <c r="B381" s="2" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>King</t>
         </is>
       </c>
       <c r="C381" s="2" t="inlineStr">
         <is>
-          <t>Tướng</t>
+          <t>Vua</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>guide.piece.advisor</t>
+          <t>guide.piece.queen</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>Advisor</t>
+          <t>Queen</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>Sĩ</t>
+          <t>Hậu</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>guide.piece.elephant</t>
+          <t>guide.piece.bishop</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>Elephant</t>
+          <t>Bishop</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
@@ -6847,12 +6847,12 @@
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>guide.piece.chariot</t>
+          <t>guide.piece.rook</t>
         </is>
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>Chariot</t>
+          <t>Rook</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
@@ -6864,12 +6864,12 @@
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>guide.piece.horse</t>
+          <t>guide.piece.knight</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>Horse</t>
+          <t>Knight</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
@@ -6881,1146 +6881,1158 @@
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>guide.piece.cannon</t>
+          <t>guide.piece.pawn</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>Cannon</t>
+          <t>Pawn</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>Pháo</t>
+          <t>Tốt</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>guide.piece.soldier</t>
+          <t>guide.moving-pieces.paragraph1</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>Soldier</t>
+          <t>Players move alternately, one legal move at a time. Piece movement rules are:</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>Tốt</t>
+          <t>Hai bên lần lượt đi quân, mỗi lượt một nước đi hợp lệ. Quy tắc di chuyển như sau:</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>guide.moving-pieces.paragraph1</t>
+          <t>guide.king.paragraph1</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>On each turn, each side may move only one of its own pieces according to the rules. The movement rules are as follows:</t>
+          <t>King</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>Mỗi nước đi, mỗi bên chỉ được di chuyển quân của mình theo đúng quy định. Quy định di chuyển của các quân như sau:</t>
+          <t>Vua</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>guide.general.paragraph1</t>
+          <t>guide.king.paragraph2</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>General</t>
+          <t>Moves one square in any direction. The King may not move into check.</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>Tướng</t>
+          <t>Di chuyển một ô theo mọi hướng. Vua không được đi vào ô đang bị chiếu.</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>guide.general.paragraph2</t>
+          <t>guide.queen.paragraph1</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>Moves one step &lt;b&gt;horizontally or vertically&lt;/b&gt; within the palace. The two Generals may not face each other directly on the same file. If they are facing each other, there must be at least one piece of either side placed between them.</t>
+          <t>Queen</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>Mỗi nước được đi một bước &lt;b&gt;ngang hoặc dọc&lt;/b&gt; tùy ý trong cung Tướng. Hai tướng của 2 bên không được đối mặt nhau trực tiếp trên cùng một đường thẳng. Nếu đối mặt, bắt buộc phải có quân của bất kỳ bên nào đứng che mặt.</t>
+          <t>Hậu</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>guide.advisor.paragraph1</t>
+          <t>guide.queen.paragraph2</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>Advisor</t>
+          <t>Moves any number of squares horizontally, vertically, or diagonally, as long as no piece blocks the path.</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>Sĩ</t>
+          <t>Di chuyển không giới hạn số ô theo hàng, cột hoặc đường chéo, miễn là không bị quân khác cản đường.</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>guide.advisor.paragraph2</t>
+          <t>guide.bishop.paragraph1</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>Moves one step &lt;b&gt;diagonally&lt;/b&gt; within the palace.</t>
+          <t>Bishop</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>Mỗi nước &lt;b&gt;đi chéo một bước&lt;/b&gt; trong cung Tướng.</t>
+          <t>Tượng</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>guide.elephant.paragraph1</t>
+          <t>guide.bishop.paragraph2</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>Elephant</t>
+          <t>Moves any number of squares diagonally and cannot jump over pieces.</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>Tượng</t>
+          <t>Di chuyển không giới hạn số ô theo đường chéo và không được nhảy qua quân khác.</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>guide.elephant.paragraph2</t>
+          <t>guide.rook.paragraph1</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;two steps diagonally&lt;/b&gt; on its own side of the board and may not cross the river. If there is another piece on the midpoint of that diagonal path, the Elephant is blocked and cannot move.</t>
+          <t>Rook</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>Mỗi nước &lt;b&gt;đi chéo hai bước&lt;/b&gt; tại trận địa bên mình, không được qua sông. Nếu ở giữa đường chéo đó có quân khác đứng thì quân Tượng bị cản, không đi được.</t>
+          <t>Xe</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>guide.chariot.paragraph1</t>
+          <t>guide.rook.paragraph2</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>Chariot</t>
+          <t>Moves any number of squares horizontally or vertically and cannot jump over pieces.</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>Xe</t>
+          <t>Di chuyển không giới hạn số ô theo hàng hoặc cột và không được nhảy qua quân khác.</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>guide.chariot.paragraph2</t>
+          <t>guide.knight.paragraph1</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; with no limit on distance, as long as no piece blocks the path.</t>
+          <t>Knight</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>Mỗi nước được &lt;b&gt;đi dọc hoặc đi ngang&lt;/b&gt;, không hạn chế số bước đi nếu không có quân khác cản đường.</t>
+          <t>Mã</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>guide.horse.paragraph1</t>
+          <t>guide.knight.paragraph2</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>Horse</t>
+          <t>Moves in an &lt;b&gt;L-shape&lt;/b&gt; (two squares in one direction and one perpendicular). The Knight can jump over pieces.</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>Mã</t>
+          <t>Di chuyển theo &lt;b&gt;hình chữ L&lt;/b&gt; (2 ô theo một hướng rồi 1 ô vuông góc). Mã có thể nhảy qua quân khác.</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>guide.horse.paragraph2</t>
+          <t>guide.pawn.paragraph1</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>Moves in an &lt;b&gt;L-shape&lt;/b&gt; (one step orthogonally then one step diagonally outward). If the adjacent orthogonal point is occupied by any piece, the Horse is blocked and cannot move.</t>
+          <t>Pawn</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>Đi theo &lt;b&gt;đường chéo hình chữ nhật&lt;/b&gt; của hai ô vuông liền nhau. Nếu giao điểm liền kề bước thẳng dọc ngang có một quân khác đứng thì Mã bị cản, không đi được.</t>
+          <t>Tốt</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>guide.cannon.paragraph1</t>
+          <t>guide.pawn.paragraph2</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>Cannon</t>
+          <t>Moves one square forward (or two squares from its starting rank if both squares are empty). Captures one square diagonally forward.</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>Pháo</t>
+          <t>Đi thẳng một ô (hoặc hai ô ở nước đi đầu tiên nếu cả hai ô đều trống). Bắt quân theo đường chéo lên trước một ô.</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>guide.cannon.paragraph2</t>
+          <t>guide.special-moves.paragraph1</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;horizontally or vertically&lt;/b&gt; like a Chariot when not capturing. To capture, it must &lt;b&gt;jump over exactly one piece&lt;/b&gt; to reach its target. If there are zero or more than one pieces between the Cannon and the target, it cannot capture.</t>
+          <t>Special Moves</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>Đi ngang hoặc dọc giống Xe khi không bắt quân. Để bắt quân, nó phải &lt;b&gt;nhảy qua đúng một quân khác&lt;/b&gt; để đến mục tiêu. Nếu không có hoặc có nhiều hơn một quân giữa Pháo và mục tiêu, nó không thể bắt quân.</t>
+          <t>Nước đi đặc biệt</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>guide.soldier.paragraph1</t>
+          <t>guide.special-moves.paragraph2</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>Soldier</t>
+          <t>&lt;b&gt;Castling&lt;/b&gt;: King moves two squares toward a rook and the rook jumps over.</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>Tốt</t>
+          <t>&lt;b&gt;Nhập thành&lt;/b&gt;: Vua đi hai ô về phía Xe và Xe nhảy qua Vua.</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>guide.soldier.paragraph2</t>
+          <t>guide.special-moves.paragraph3</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>Moves &lt;b&gt;one step&lt;/b&gt; each turn. Before crossing the river, it can only move forward. After crossing the river, it may move &lt;b&gt;forward or sideways&lt;/b&gt;, but never backward.</t>
+          <t>&lt;b&gt;En passant&lt;/b&gt;: special pawn capture &lt;b&gt;right after&lt;/b&gt; an opponent pawn advances two squares.</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
         <is>
-          <t>Mỗi nước đi &lt;b&gt;một bước&lt;/b&gt;. Khi chưa qua sông, Tốt chỉ được tiến. Khi Tốt đã qua sông được quyền &lt;b&gt;đi tiến và đi ngang&lt;/b&gt;, không được phép lùi.</t>
+          <t>&lt;b&gt;Bắt tốt qua đường&lt;/b&gt; (en passant): bắt tốt đối phương &lt;b&gt;ngay sau khi&lt;/b&gt; tốt đó đi hai ô.</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>guide.capturing.paragraph1</t>
+          <t>guide.special-moves.paragraph4</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>When a piece moves to an intersection occupied by an opponent's piece, it may &lt;b&gt;capture that piece&lt;/b&gt; and occupy its position.</t>
+          <t>&lt;b&gt;Promotion&lt;/b&gt;: when a pawn reaches the last rank, it promotes to Queen, Rook, Bishop, or Knight.</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
         <is>
-          <t>Khi một quân đi tới một giao điểm khác đã có quân đối phương đứng thì được quyền &lt;b&gt;bắt quân đó&lt;/b&gt;, đồng thời chiếm giữ vị trí quân bị bắt.</t>
+          <t>&lt;b&gt;Phong cấp&lt;/b&gt;: khi Tốt tới hàng cuối, được phong thành Hậu, Xe, Tượng hoặc Mã.</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>guide.capturing.paragraph2</t>
+          <t>guide.capturing.paragraph1</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>You may not capture your own pieces. You may sacrifice your own pieces to be captured by the opponent, &lt;b&gt;except for the General&lt;/b&gt;.</t>
+          <t>A piece captures by moving to a square occupied by an opponent piece. Captured pieces are removed from the board.</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t>Không được bắt quân bên mình. Được phép cho đối phương bắt đầu quân mình chủ động hiến mình cho đối phương, &lt;b&gt;trừ Tướng&lt;/b&gt;.</t>
+          <t>Quân cờ bắt bằng cách đi đến ô có quân đối phương. Quân bị bắt sẽ bị loại khỏi bàn cờ.</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>guide.capturing.paragraph3</t>
+          <t>guide.capturing.paragraph2</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>A captured piece is removed from the board. &lt;b&gt;Chasing one piece for more than 6 consecutive moves is not allowed&lt;/b&gt;.</t>
+          <t>You cannot capture your own pieces. Except for the Knight, pieces cannot jump over other pieces.</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t>Quân bị bắt phải bị loại và bị nhấc ra khỏi bàn cờ. &lt;b&gt;Không được đuổi 1 quân quá 6 nước cờ liên tiếp&lt;/b&gt;.</t>
+          <t>Không được bắt quân của chính mình. Trừ Mã, các quân khác không được nhảy qua quân cờ.</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>guide.check.paragraph1</t>
+          <t>guide.capturing.paragraph3</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>If a player makes a move that threatens to capture the opponent's General on the next move (by the same piece or another piece), it is called a &lt;b&gt;Check&lt;/b&gt;. The checked side must respond to avoid check. Otherwise, that side loses</t>
+          <t>The King is never captured. The game is won by checkmate, or ends by resignation/draw.</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t>Nếu người chơi thực hiện một nước đi đe dọa bắt Tướng của đối phương ở nước đi tiếp theo (bằng chính quân cờ đó hoặc một quân cờ khác), thì đó được gọi là &lt;b&gt;Chiếu&lt;/b&gt;. Bên bị chiếu phải đáp trả để tránh bị chiếu. Nếu không sẽ bị xử thua</t>
+          <t>Vua không bao giờ bị bắt trực tiếp. Ván cờ thắng bằng chiếu bí, hoặc kết thúc bằng đầu hàng/hòa.</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>guide.check.paragraph2</t>
+          <t>guide.check.paragraph1</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>When the General is checked from any direction (including from behind), the checked side may respond in one of the following ways:</t>
+          <t>A King is in &lt;b&gt;check&lt;/b&gt; when attacked by one or more opponent pieces. You must respond immediately.</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t>Tướng bị chiếu từ cả bốn hướng (bị chiếu cả từ phía sau) có thể ứng phó với nước chiếu tướng bằng một trong các cách sau:</t>
+          <t>&lt;b&gt;Chiếu&lt;/b&gt; là khi Vua bị một hoặc nhiều quân đối phương tấn công. Bên bị chiếu phải xử lý ngay.</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>guide.check.paragraph3</t>
+          <t>guide.check.paragraph2</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>Move the General to another position to escape check</t>
+          <t>To respond to check, a player may choose one of the following legal options:</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
         <is>
-          <t>Di chuyển tướng sang vị trí khác để tránh nước chiếu</t>
+          <t>Để thoát chiếu, người chơi có thể chọn một trong các cách hợp lệ sau:</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>guide.check.paragraph4</t>
+          <t>guide.check.paragraph3</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>Capture the checking piece</t>
+          <t>Move the King to a safe square</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
         <is>
-          <t>Bắt quân đang chiếu</t>
+          <t>Di chuyển Vua đến ô an toàn</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>guide.check.paragraph5</t>
+          <t>guide.check.paragraph4</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>Block the checking line with another piece to protect the General</t>
+          <t>Capture the attacking piece</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>Dùng quân khác cản quân chiếu, đi quân che đỡ cho tướng</t>
+          <t>Bắt quân đang chiếu</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>guide.check.paragraph6</t>
+          <t>guide.check.paragraph5</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>Repeatedly checking for more than 6 consecutive moves is not allowed</t>
+          <t>Block the line of attack (if possible)</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
         <is>
-          <t>Không được chiếu tướng quá 6 nước cờ liên tiếp</t>
+          <t>Chặn đường chiếu (nếu có thể)</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>guide.result.paragraph1</t>
+          <t>guide.check.paragraph6</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>When one side gives Check and the other side has no legal way to protect the General, it is called a &lt;b&gt;Checkmate&lt;/b&gt;. The side that delivers Checkmate wins.</t>
+          <t>If none of these is possible, it is checkmate and the game is lost.</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
         <is>
-          <t>Khi một bên chiếu Tướng mà bên còn lại không thể làm gì để bảo vệ Tướng thì được gọi là &lt;b&gt;Chiếu Hết&lt;/b&gt;, bên thực hiện được Chiếu Hết sẽ giành chiến thắng.</t>
+          <t>Nếu không thể làm cách nào ở trên, đó là chiếu bí và ván cờ kết thúc thua.</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>guide.result.paragraph2</t>
+          <t>guide.result.paragraph1</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>If a player runs out of time for a single move (for example: 90s) without moving, the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
+          <t>A game is won by &lt;b&gt;checkmate&lt;/b&gt;, when the checked King has no legal escape.</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>Khi hết thời gian một nước đi (ví dụ: 90s) mà vẫn chưa di chuyển quân thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
+          <t>Ván cờ thắng bằng &lt;b&gt;chiếu bí&lt;/b&gt;, khi Vua bị chiếu và không còn nước hợp lệ để thoát.</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>guide.result.paragraph3</t>
+          <t>guide.result.paragraph2</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>If a player runs out of total game time (for example: 5 minutes or 10 minutes), the other side is awarded a &lt;b&gt;win&lt;/b&gt;.</t>
+          <t>If a player runs out of move time (in modes that use per-move time), that player loses.</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t>Khi một bên hết thời gian ván đấu (ví dụ: 5 phút, 10 phút) thì bên còn lại sẽ được &lt;b&gt;xử Thắng&lt;/b&gt;.</t>
+          <t>Nếu người chơi hết thời gian cho một nước đi (ở chế độ có giới hạn thời gian mỗi nước), người đó thua.</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>guide.result.paragraph4</t>
+          <t>guide.result.paragraph3</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>If both sides have no pieces that have crossed the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;. If one side still has pieces across the river but runs out of time, while the other side still has time but has no pieces across the river, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
+          <t>If a player runs out of total game time, that player loses (unless the opponent has no possible mating sequence).</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t>Khi cả 2 bên đều không còn quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;. Khi một bên còn quân qua sông nhưng cạn thời gian, một bên còn thời gian nhưng hết quân qua sông, ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
+          <t>Nếu người chơi hết tổng thời gian ván đấu, người đó thua (trừ khi đối phương không còn khả năng chiếu bí bằng bất kỳ chuỗi nước hợp lệ nào).</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>guide.result.paragraph5</t>
+          <t>guide.result.paragraph4</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>Within 50 moves, if there is no capture and no Soldier advances by one square, the game is declared a &lt;b&gt;draw&lt;/b&gt;.</t>
+          <t>A game is drawn by stalemate, dead position (insufficient mating material), or draw agreement.</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t>Trong vòng 50 nước nếu không phát sinh nước bắt quân, Tốt không tiến 1 ô thì ván đấu sẽ được &lt;b&gt;xử Hòa&lt;/b&gt;.</t>
+          <t>Ván cờ hòa khi rơi vào thế bí không bị chiếu (stalemate), thế chết (không đủ lực chiếu bí), hoặc hai bên đồng ý hòa.</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>extra-money.title</t>
+          <t>guide.result.paragraph5</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>Daily tasks</t>
+          <t>A game can also be drawn by the &lt;b&gt;50-move rule&lt;/b&gt; or &lt;b&gt;threefold repetition&lt;/b&gt; according to the rules.</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
         <is>
-          <t>Kiếm tiền</t>
+          <t>Ván cờ cũng có thể hòa theo &lt;b&gt;luật 50 nước&lt;/b&gt; hoặc &lt;b&gt;lặp lại vị trí 3 lần&lt;/b&gt; theo luật.</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>extra-money.tab.lucky-wheel</t>
+          <t>extra-money.title</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>Lucky Wheel</t>
+          <t>Daily tasks</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
         <is>
-          <t>Vòng Quay May Mắn</t>
+          <t>Kiếm tiền</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>extra-money.tab.bonus-coin</t>
+          <t>extra-money.tab.lucky-wheel</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>Bonus Coin</t>
+          <t>Lucky Wheel</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
         <is>
-          <t>Xu Thưởng</t>
+          <t>Vòng Quay May Mắn</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>extra-money.tab.daily-bonus</t>
+          <t>extra-money.tab.bonus-coin</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>Daily Bonus</t>
+          <t>Bonus Coin</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
         <is>
-          <t>Thưởng hàng ngày</t>
+          <t>Xu Thưởng</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.subtitle</t>
+          <t>extra-money.tab.daily-bonus</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>Watch a short video to earn free coin</t>
+          <t>Daily Bonus</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>Xem video ngắn để nhận xu miễn phí</t>
+          <t>Thưởng hàng ngày</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.next-in</t>
+          <t>extra-money.bonus-coin.subtitle</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>Next in:</t>
+          <t>Watch a short video to earn free coin</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t>Lượt kế tiếp:</t>
+          <t>Xem video ngắn để nhận xu miễn phí</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.collect</t>
+          <t>extra-money.bonus-coin.next-in</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>Collect</t>
+          <t>Next in:</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t>Thu thập</t>
+          <t>Lượt kế tiếp:</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>extra-money.bonus-coin.watch-video</t>
+          <t>extra-money.bonus-coin.collect</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>Watch video</t>
+          <t>Collect</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t>Xem video</t>
+          <t>Thu thập</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>extra-money.daily-bonus.subtitle</t>
+          <t>extra-money.bonus-coin.watch-video</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>Login 7 days in a row to earn 4000 coin</t>
+          <t>Watch video</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t>Đăng nhập 7 ngày liên tiếp để nhận 4000 xu</t>
+          <t>Xem video</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>extra-money.daily-bonus.day</t>
+          <t>extra-money.daily-bonus.subtitle</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>Day</t>
+          <t>Login 7 days in a row to earn 4000 coin</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
         <is>
-          <t>Ngày</t>
+          <t>Đăng nhập 7 ngày liên tiếp để nhận 4000 xu</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.loading</t>
+          <t>extra-money.daily-bonus.day</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>Loading ad...</t>
+          <t>Day</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
         <is>
-          <t>Đang tải quảng cáo...</t>
+          <t>Ngày</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.error</t>
+          <t>extra-money.reward-ad.loading</t>
         </is>
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>Could not load the ad. Please try again.</t>
+          <t>Loading ad...</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
         <is>
-          <t>Không tải được quảng cáo. Vui lòng thử lại.</t>
+          <t>Đang tải quảng cáo...</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.retry</t>
+          <t>extra-money.reward-ad.error</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>Try again</t>
+          <t>Could not load the ad. Please try again.</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
         <is>
-          <t>Thử lại</t>
+          <t>Không tải được quảng cáo. Vui lòng thử lại.</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>extra-money.reward-ad.close</t>
+          <t>extra-money.reward-ad.retry</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>Close</t>
+          <t>Try again</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
         <is>
-          <t>Đóng</t>
+          <t>Thử lại</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>profile.button.save</t>
+          <t>extra-money.reward-ad.close</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>Save</t>
+          <t>Close</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
         <is>
-          <t>Lưu</t>
+          <t>Đóng</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>profile.button.cancel</t>
+          <t>profile.button.save</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>Cancel</t>
+          <t>Save</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
         <is>
-          <t>Huỷ</t>
+          <t>Lưu</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>change-password.title</t>
+          <t>profile.button.cancel</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>Change password</t>
+          <t>Cancel</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
         <is>
-          <t>Đổi mật khẩu</t>
+          <t>Huỷ</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>change-password.current.label</t>
+          <t>change-password.title</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>Current password</t>
+          <t>Change password</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
         <is>
-          <t>Mật khẩu hiện tại</t>
+          <t>Đổi mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>change-password.current.placeholder</t>
+          <t>change-password.current.label</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>Enter current password</t>
+          <t>Current password</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
         <is>
-          <t>Nhập mật khẩu hiện tại</t>
+          <t>Mật khẩu hiện tại</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>change-password.new.label</t>
+          <t>change-password.current.placeholder</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>New password</t>
+          <t>Enter current password</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
         <is>
-          <t>Mật khẩu mới</t>
+          <t>Nhập mật khẩu hiện tại</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>change-password.new.placeholder</t>
+          <t>change-password.new.label</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>Enter new password</t>
+          <t>New password</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
         <is>
-          <t>Nhập mật khẩu mới</t>
+          <t>Mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>change-password.confirm.label</t>
+          <t>change-password.new.placeholder</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>Confirm new password</t>
+          <t>Enter new password</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>Xác nhận mật khẩu mới</t>
+          <t>Nhập mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>change-password.confirm.placeholder</t>
+          <t>change-password.confirm.label</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>Re-enter new password</t>
+          <t>Confirm new password</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
         <is>
-          <t>Nhập lại mật khẩu mới</t>
+          <t>Xác nhận mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>change-password.confirm.mismatch</t>
+          <t>change-password.confirm.placeholder</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>Passwords do not match</t>
+          <t>Re-enter new password</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t>Mật khẩu xác nhận không khớp</t>
+          <t>Nhập lại mật khẩu mới</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>change-password.show</t>
+          <t>change-password.confirm.mismatch</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>Show password</t>
+          <t>Passwords do not match</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t>Hiện mật khẩu</t>
+          <t>Mật khẩu xác nhận không khớp</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>change-password.hide</t>
+          <t>change-password.show</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>Hide password</t>
+          <t>Show password</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>Ẩn mật khẩu</t>
+          <t>Hiện mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>change-password.submit</t>
+          <t>change-password.hide</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>Change password</t>
+          <t>Hide password</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>Đổi mật khẩu</t>
+          <t>Ẩn mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>change-password.submitting</t>
+          <t>change-password.submit</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>Changing...</t>
+          <t>Change password</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>Đang đổi...</t>
+          <t>Đổi mật khẩu</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>change-password.messages.success</t>
+          <t>change-password.submitting</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>Password changed successfully</t>
+          <t>Changing...</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>Đổi mật khẩu thành công</t>
+          <t>Đang đổi...</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>change-password.messages.missing-fields</t>
+          <t>change-password.messages.success</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>Please fill in all fields</t>
+          <t>Password changed successfully</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
         <is>
-          <t>Vui lòng nhập đầy đủ thông tin</t>
+          <t>Đổi mật khẩu thành công</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>change-password.messages.weak-password</t>
+          <t>change-password.messages.missing-fields</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>New password does not meet the requirements</t>
+          <t>Please fill in all fields</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
         <is>
-          <t>Mật khẩu mới không đạt yêu cầu</t>
+          <t>Vui lòng nhập đầy đủ thông tin</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>change-password.messages.same-as-current</t>
+          <t>change-password.messages.weak-password</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>New password must be different from the current one</t>
+          <t>New password does not meet the requirements</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
         <is>
-          <t>Mật khẩu mới phải khác mật khẩu hiện tại</t>
+          <t>Mật khẩu mới không đạt yêu cầu</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>change-password.messages.incorrect-current-password</t>
+          <t>change-password.messages.same-as-current</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>Current password is incorrect</t>
+          <t>New password must be different from the current one</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
         <is>
-          <t>Mật khẩu hiện tại không đúng</t>
+          <t>Mật khẩu mới phải khác mật khẩu hiện tại</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>change-password.messages.user-not-found</t>
+          <t>change-password.messages.incorrect-current-password</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>User not found</t>
+          <t>Current password is incorrect</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
         <is>
-          <t>Không tìm thấy người dùng</t>
+          <t>Mật khẩu hiện tại không đúng</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>change-password.messages.unauthorized</t>
+          <t>change-password.messages.user-not-found</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>Session expired. Please sign in again.</t>
+          <t>User not found</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>Phiên đăng nhập đã hết hạn. Vui lòng đăng nhập lại.</t>
+          <t>Không tìm thấy người dùng</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
+          <t>change-password.messages.unauthorized</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Session expired. Please sign in again.</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Phiên đăng nhập đã hết hạn. Vui lòng đăng nhập lại.</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
           <t>change-password.messages.internal-server-error</t>
         </is>
       </c>
-      <c r="B452" t="inlineStr">
+      <c r="B453" t="inlineStr">
         <is>
           <t>Something went wrong. Please try again.</t>
         </is>
       </c>
-      <c r="C452" t="inlineStr">
+      <c r="C453" t="inlineStr">
         <is>
           <t>Đã có lỗi xảy ra. Vui lòng thử lại.</t>
         </is>
       </c>
-    </row>
-    <row r="453">
-      <c r="A453" t="inlineStr"/>
-      <c r="B453" t="inlineStr"/>
-      <c r="C453" t="inlineStr"/>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr"/>
@@ -8111,6 +8123,11 @@
       <c r="A471" t="inlineStr"/>
       <c r="B471" t="inlineStr"/>
       <c r="C471" t="inlineStr"/>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr"/>
+      <c r="B472" t="inlineStr"/>
+      <c r="C472" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>